<commit_message>
Fixed failed scenarios and Removed unnecessary imports
Fixed failed scenarios and Removed unnecessary imports
</commit_message>
<xml_diff>
--- a/testdata/DirectGRN-FOC Scenarios.xlsx
+++ b/testdata/DirectGRN-FOC Scenarios.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1564" uniqueCount="167">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -488,6 +488,54 @@
   </si>
   <si>
     <t>GWL-RM-WAL-01 PriceList-DIS-UOM</t>
+  </si>
+  <si>
+    <t>20000.5</t>
+  </si>
+  <si>
+    <t>232</t>
+  </si>
+  <si>
+    <t>16638.94611</t>
+  </si>
+  <si>
+    <t>60001.5</t>
+  </si>
+  <si>
+    <t>34.684</t>
+  </si>
+  <si>
+    <t>59017.31249</t>
+  </si>
+  <si>
+    <t>17000</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>16698.11321</t>
+  </si>
+  <si>
+    <t>51000</t>
+  </si>
+  <si>
+    <t>36.682</t>
+  </si>
+  <si>
+    <t>50045.49914</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>16672.13116</t>
+  </si>
+  <si>
+    <t>39.35</t>
+  </si>
+  <si>
+    <t>50008.51333</t>
   </si>
 </sst>
 </file>
@@ -1877,7 +1925,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -2177,8 +2225,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -2195,8 +2243,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -2265,8 +2313,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -2283,8 +2331,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -2353,8 +2401,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -2371,8 +2419,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -2441,8 +2489,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -2459,8 +2507,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -2529,8 +2577,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -2547,8 +2595,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -2617,8 +2665,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -2635,8 +2683,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -2705,8 +2753,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -2723,8 +2771,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -2793,8 +2841,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -2811,8 +2859,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -2881,8 +2929,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -2899,8 +2947,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -2969,8 +3017,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -2987,8 +3035,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -3057,8 +3105,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -3075,8 +3123,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -3145,8 +3193,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -3163,8 +3211,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -3233,8 +3281,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -3251,8 +3299,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -3321,8 +3369,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -3339,8 +3387,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -3409,8 +3457,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -3427,8 +3475,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -3485,8 +3533,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -3503,8 +3551,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -3816,12 +3864,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -3870,12 +3914,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -4050,8 +4090,12 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47"/>
-      <c r="AV23" s="47"/>
+      <c r="AU23" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="AV23" t="s" s="0">
+        <v>151</v>
+      </c>
       <c r="AW23" s="50">
         <f>AM23</f>
         <v>2</v>
@@ -4090,11 +4134,11 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>120</v>
+      <c r="BM23" t="s" s="0">
+        <v>153</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>152</v>
       </c>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -4249,8 +4293,8 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="16.0"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -4550,8 +4594,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -4568,8 +4612,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -4638,8 +4682,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -4656,8 +4700,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -4726,8 +4770,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -4744,8 +4788,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -4814,8 +4858,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -4832,8 +4876,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -4902,8 +4946,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -4920,8 +4964,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -4990,8 +5034,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -5008,8 +5052,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -5078,8 +5122,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -5096,8 +5140,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -5166,8 +5210,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -5184,8 +5228,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -5254,8 +5298,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -5272,8 +5316,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -5342,8 +5386,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -5360,8 +5404,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -5430,8 +5474,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -5448,8 +5492,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -5518,8 +5562,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -5536,8 +5580,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -5606,8 +5650,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -5624,8 +5668,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -5694,8 +5738,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -5712,8 +5756,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -5782,8 +5826,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -5800,8 +5844,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -5858,8 +5902,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -5876,8 +5920,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -6189,12 +6233,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -6243,12 +6283,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -6423,12 +6459,8 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
-        <v>112</v>
-      </c>
-      <c r="AV23" s="47" t="s">
-        <v>124</v>
-      </c>
+      <c r="AU23" s="0"/>
+      <c r="AV23" s="0"/>
       <c r="AW23" s="50">
         <f>AM23</f>
         <v>2</v>
@@ -6467,12 +6499,8 @@
       <c r="BL23" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>127</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>128</v>
-      </c>
+      <c r="BM23" s="0"/>
+      <c r="BN23" s="0"/>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>277.52168</v>
@@ -6626,7 +6654,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -6926,8 +6954,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -6944,8 +6972,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -7014,8 +7042,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -7032,8 +7060,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -7102,8 +7130,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -7120,8 +7148,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -7190,8 +7218,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -7208,8 +7236,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -7278,8 +7306,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -7296,8 +7324,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -7366,8 +7394,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -7384,8 +7412,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -7454,8 +7482,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -7472,8 +7500,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -7542,8 +7570,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -7560,8 +7588,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -7630,8 +7658,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -7648,8 +7676,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -7718,8 +7746,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -7736,8 +7764,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -7806,8 +7834,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -7824,8 +7852,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -7894,8 +7922,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -7912,8 +7940,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -7982,8 +8010,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -8000,8 +8028,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -8070,8 +8098,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -8088,8 +8116,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -8158,8 +8186,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -8176,8 +8204,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -8234,8 +8262,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -8252,8 +8280,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -8565,12 +8593,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -8619,12 +8643,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -8654,14 +8674,14 @@
       <c r="F23" s="28">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
       <c r="H23" s="28">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>120</v>
       </c>
       <c r="J23" s="28">
@@ -8799,11 +8819,11 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
+      <c r="AU23" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="AV23" s="47" t="s">
-        <v>131</v>
+      <c r="AV23" t="s" s="0">
+        <v>157</v>
       </c>
       <c r="AW23" s="50">
         <f>AM23</f>
@@ -8843,11 +8863,11 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>132</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>133</v>
+      <c r="BM23" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>158</v>
       </c>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -9002,7 +9022,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -9302,8 +9322,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -9320,8 +9340,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -9390,8 +9410,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -9408,8 +9428,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -9478,8 +9498,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -9496,8 +9516,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -9566,8 +9586,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -9584,8 +9604,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -9654,8 +9674,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -9672,8 +9692,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -9742,8 +9762,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -9760,8 +9780,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -9830,8 +9850,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -9848,8 +9868,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -9918,8 +9938,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -9936,8 +9956,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -10006,8 +10026,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -10024,8 +10044,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -10094,8 +10114,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -10112,8 +10132,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -10182,8 +10202,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -10200,8 +10220,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -10270,8 +10290,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -10288,8 +10308,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -10358,8 +10378,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -10376,8 +10396,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -10446,8 +10466,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -10464,8 +10484,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -10534,8 +10554,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -10552,8 +10572,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -10610,8 +10630,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -10628,8 +10648,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -10941,12 +10961,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -10995,12 +11011,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -11030,14 +11042,14 @@
       <c r="F23" s="28">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
       <c r="H23" s="28">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>120</v>
       </c>
       <c r="J23" s="28">
@@ -11175,12 +11187,8 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
-        <v>135</v>
-      </c>
-      <c r="AV23" s="47" t="s">
-        <v>136</v>
-      </c>
+      <c r="AU23" s="0"/>
+      <c r="AV23" s="0"/>
       <c r="AW23" s="50">
         <f>AM23</f>
         <v>2</v>
@@ -11219,12 +11227,8 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>137</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>138</v>
-      </c>
+      <c r="BM23" s="0"/>
+      <c r="BN23" s="0"/>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>146.93407</v>
@@ -11372,7 +11376,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -11672,8 +11676,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -11690,8 +11694,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -11760,8 +11764,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -11778,8 +11782,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -11848,8 +11852,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -11866,8 +11870,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -11936,8 +11940,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -11954,8 +11958,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -12024,8 +12028,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -12042,8 +12046,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -12112,8 +12116,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -12130,8 +12134,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -12200,8 +12204,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -12218,8 +12222,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -12288,8 +12292,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -12306,8 +12310,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -12376,8 +12380,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -12394,8 +12398,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -12464,8 +12468,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -12482,8 +12486,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -12552,8 +12556,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -12570,8 +12574,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -12640,8 +12644,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -12658,8 +12662,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -12728,8 +12732,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -12746,8 +12750,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -12816,8 +12820,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -12834,8 +12838,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -12904,8 +12908,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -12922,8 +12926,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -12980,8 +12984,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -12998,8 +13002,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -13311,12 +13315,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -13365,12 +13365,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -13400,14 +13396,14 @@
       <c r="F23" s="28">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
       <c r="H23" s="28">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>120</v>
       </c>
       <c r="J23" s="28">
@@ -13545,11 +13541,11 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
+      <c r="AU23" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="AV23" s="47" t="s">
-        <v>140</v>
+      <c r="AV23" t="s" s="0">
+        <v>157</v>
       </c>
       <c r="AW23" s="50">
         <f>AM23</f>
@@ -13589,11 +13585,11 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>140</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>141</v>
+      <c r="BM23" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>163</v>
       </c>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -14045,8 +14041,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -14063,8 +14059,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -14133,8 +14129,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -14151,8 +14147,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -14221,8 +14217,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -14239,8 +14235,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -14309,8 +14305,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -14327,8 +14323,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -14397,8 +14393,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -14415,8 +14411,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -14485,8 +14481,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -14503,8 +14499,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -14573,8 +14569,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -14591,8 +14587,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -14661,8 +14657,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -14679,8 +14675,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -14749,8 +14745,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -14767,8 +14763,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -14837,8 +14833,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -14855,8 +14851,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -14925,8 +14921,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -14943,8 +14939,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -15013,8 +15009,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -15031,8 +15027,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -15101,8 +15097,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -15119,8 +15115,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -15189,8 +15185,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -15207,8 +15203,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -15277,8 +15273,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -15295,8 +15291,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -15353,8 +15349,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -15371,8 +15367,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -15684,12 +15680,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -15738,12 +15730,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -15773,14 +15761,14 @@
       <c r="F23" s="28">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
       <c r="H23" s="28">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>120</v>
       </c>
       <c r="J23" s="28">
@@ -15918,12 +15906,8 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
-        <v>143</v>
-      </c>
-      <c r="AV23" s="47" t="s">
-        <v>144</v>
-      </c>
+      <c r="AU23" s="0"/>
+      <c r="AV23" s="0"/>
       <c r="AW23" s="50">
         <f>AM23</f>
         <v>2</v>
@@ -15962,12 +15946,8 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>145</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>146</v>
-      </c>
+      <c r="BM23" s="0"/>
+      <c r="BN23" s="0"/>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>184.84725</v>
@@ -16121,7 +16101,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -16421,8 +16401,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -16439,8 +16419,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -16509,8 +16489,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -16527,8 +16507,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -16597,8 +16577,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -16615,8 +16595,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -16685,8 +16665,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -16703,8 +16683,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -16773,8 +16753,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -16791,8 +16771,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -16861,8 +16841,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -16879,8 +16859,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -16949,8 +16929,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -16967,8 +16947,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -17037,8 +17017,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -17055,8 +17035,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -17125,8 +17105,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -17143,8 +17123,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -17213,8 +17193,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -17231,8 +17211,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -17301,8 +17281,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -17319,8 +17299,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -17389,8 +17369,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -17407,8 +17387,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -17477,8 +17457,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -17495,8 +17475,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -17565,8 +17545,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -17583,8 +17563,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -17653,8 +17633,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -17671,8 +17651,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -17729,8 +17709,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -17747,8 +17727,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -18060,12 +18040,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -18114,12 +18090,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -18294,8 +18266,12 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47"/>
-      <c r="AV23" s="47"/>
+      <c r="AU23" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="AV23" t="s" s="0">
+        <v>154</v>
+      </c>
       <c r="AW23" s="50">
         <f>AM23</f>
         <v>0.666666666666667</v>
@@ -18334,11 +18310,11 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>120</v>
+      <c r="BM23" t="s" s="0">
+        <v>156</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>155</v>
       </c>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -18493,8 +18469,8 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.5727272727273" customWidth="1"/>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.5727272727273"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -18794,8 +18770,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -18812,8 +18788,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -18882,8 +18858,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -18900,8 +18876,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -18970,8 +18946,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -18988,8 +18964,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -19058,8 +19034,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -19076,8 +19052,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -19146,8 +19122,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -19164,8 +19140,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -19234,8 +19210,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -19252,8 +19228,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -19322,8 +19298,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -19340,8 +19316,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -19410,8 +19386,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -19428,8 +19404,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -19498,8 +19474,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -19516,8 +19492,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -19586,8 +19562,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -19604,8 +19580,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -19674,8 +19650,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -19692,8 +19668,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -19762,8 +19738,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -19780,8 +19756,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -19850,8 +19826,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -19868,8 +19844,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -19938,8 +19914,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -19956,8 +19932,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -20026,8 +20002,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -20044,8 +20020,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -20102,8 +20078,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -20120,8 +20096,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -20433,12 +20409,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -20487,12 +20459,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -20522,14 +20490,14 @@
       <c r="F23" s="28">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
       <c r="H23" s="28">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>120</v>
       </c>
       <c r="J23" s="28">
@@ -20667,11 +20635,11 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
+      <c r="AU23" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="AV23" s="47" t="s">
-        <v>131</v>
+      <c r="AV23" t="s" s="0">
+        <v>160</v>
       </c>
       <c r="AW23" s="50">
         <f>AM23</f>
@@ -20711,11 +20679,11 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>132</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>133</v>
+      <c r="BM23" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>161</v>
       </c>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -20870,7 +20838,7 @@
   <dimension ref="A1:BQ24"/>
   <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="8" max="8" width="9.42727272727273" customWidth="1"/>
+    <col min="8" max="8" customWidth="true" width="9.42727272727273"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:69">
@@ -21170,8 +21138,8 @@
       <c r="AR4" s="34"/>
       <c r="AS4" s="16"/>
       <c r="AT4" s="47"/>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
+      <c r="AU4" s="0"/>
+      <c r="AV4" s="0"/>
       <c r="AW4" s="47"/>
       <c r="AX4" s="47"/>
       <c r="AY4" s="47"/>
@@ -21188,8 +21156,8 @@
       <c r="BJ4" s="47"/>
       <c r="BK4" s="47"/>
       <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="47"/>
+      <c r="BM4" s="0"/>
+      <c r="BN4" s="0"/>
       <c r="BO4" s="47"/>
       <c r="BP4" s="47"/>
       <c r="BQ4" s="47"/>
@@ -21258,8 +21226,8 @@
       <c r="AR5" s="34"/>
       <c r="AS5" s="16"/>
       <c r="AT5" s="47"/>
-      <c r="AU5" s="47"/>
-      <c r="AV5" s="47"/>
+      <c r="AU5" s="0"/>
+      <c r="AV5" s="0"/>
       <c r="AW5" s="47"/>
       <c r="AX5" s="47"/>
       <c r="AY5" s="47"/>
@@ -21276,8 +21244,8 @@
       <c r="BJ5" s="47"/>
       <c r="BK5" s="47"/>
       <c r="BL5" s="47"/>
-      <c r="BM5" s="47"/>
-      <c r="BN5" s="47"/>
+      <c r="BM5" s="0"/>
+      <c r="BN5" s="0"/>
       <c r="BO5" s="47"/>
       <c r="BP5" s="47"/>
       <c r="BQ5" s="47"/>
@@ -21346,8 +21314,8 @@
       <c r="AR6" s="34"/>
       <c r="AS6" s="16"/>
       <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
+      <c r="AU6" s="0"/>
+      <c r="AV6" s="0"/>
       <c r="AW6" s="47"/>
       <c r="AX6" s="47"/>
       <c r="AY6" s="47"/>
@@ -21364,8 +21332,8 @@
       <c r="BJ6" s="47"/>
       <c r="BK6" s="47"/>
       <c r="BL6" s="47"/>
-      <c r="BM6" s="47"/>
-      <c r="BN6" s="47"/>
+      <c r="BM6" s="0"/>
+      <c r="BN6" s="0"/>
       <c r="BO6" s="47"/>
       <c r="BP6" s="47"/>
       <c r="BQ6" s="47"/>
@@ -21434,8 +21402,8 @@
       <c r="AR7" s="34"/>
       <c r="AS7" s="16"/>
       <c r="AT7" s="47"/>
-      <c r="AU7" s="47"/>
-      <c r="AV7" s="47"/>
+      <c r="AU7" s="0"/>
+      <c r="AV7" s="0"/>
       <c r="AW7" s="47"/>
       <c r="AX7" s="47"/>
       <c r="AY7" s="47"/>
@@ -21452,8 +21420,8 @@
       <c r="BJ7" s="47"/>
       <c r="BK7" s="47"/>
       <c r="BL7" s="47"/>
-      <c r="BM7" s="47"/>
-      <c r="BN7" s="47"/>
+      <c r="BM7" s="0"/>
+      <c r="BN7" s="0"/>
       <c r="BO7" s="47"/>
       <c r="BP7" s="47"/>
       <c r="BQ7" s="47"/>
@@ -21522,8 +21490,8 @@
       <c r="AR8" s="34"/>
       <c r="AS8" s="16"/>
       <c r="AT8" s="47"/>
-      <c r="AU8" s="47"/>
-      <c r="AV8" s="47"/>
+      <c r="AU8" s="0"/>
+      <c r="AV8" s="0"/>
       <c r="AW8" s="47"/>
       <c r="AX8" s="47"/>
       <c r="AY8" s="47"/>
@@ -21540,8 +21508,8 @@
       <c r="BJ8" s="47"/>
       <c r="BK8" s="47"/>
       <c r="BL8" s="47"/>
-      <c r="BM8" s="47"/>
-      <c r="BN8" s="47"/>
+      <c r="BM8" s="0"/>
+      <c r="BN8" s="0"/>
       <c r="BO8" s="47"/>
       <c r="BP8" s="47"/>
       <c r="BQ8" s="47"/>
@@ -21610,8 +21578,8 @@
       <c r="AR9" s="34"/>
       <c r="AS9" s="16"/>
       <c r="AT9" s="47"/>
-      <c r="AU9" s="47"/>
-      <c r="AV9" s="47"/>
+      <c r="AU9" s="0"/>
+      <c r="AV9" s="0"/>
       <c r="AW9" s="47"/>
       <c r="AX9" s="47"/>
       <c r="AY9" s="47"/>
@@ -21628,8 +21596,8 @@
       <c r="BJ9" s="47"/>
       <c r="BK9" s="47"/>
       <c r="BL9" s="47"/>
-      <c r="BM9" s="47"/>
-      <c r="BN9" s="47"/>
+      <c r="BM9" s="0"/>
+      <c r="BN9" s="0"/>
       <c r="BO9" s="47"/>
       <c r="BP9" s="47"/>
       <c r="BQ9" s="47"/>
@@ -21698,8 +21666,8 @@
       <c r="AR10" s="34"/>
       <c r="AS10" s="16"/>
       <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
+      <c r="AU10" s="0"/>
+      <c r="AV10" s="0"/>
       <c r="AW10" s="47"/>
       <c r="AX10" s="47"/>
       <c r="AY10" s="47"/>
@@ -21716,8 +21684,8 @@
       <c r="BJ10" s="47"/>
       <c r="BK10" s="47"/>
       <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="47"/>
+      <c r="BM10" s="0"/>
+      <c r="BN10" s="0"/>
       <c r="BO10" s="47"/>
       <c r="BP10" s="47"/>
       <c r="BQ10" s="47"/>
@@ -21786,8 +21754,8 @@
       <c r="AR11" s="34"/>
       <c r="AS11" s="16"/>
       <c r="AT11" s="47"/>
-      <c r="AU11" s="47"/>
-      <c r="AV11" s="47"/>
+      <c r="AU11" s="0"/>
+      <c r="AV11" s="0"/>
       <c r="AW11" s="47"/>
       <c r="AX11" s="47"/>
       <c r="AY11" s="47"/>
@@ -21804,8 +21772,8 @@
       <c r="BJ11" s="47"/>
       <c r="BK11" s="47"/>
       <c r="BL11" s="47"/>
-      <c r="BM11" s="47"/>
-      <c r="BN11" s="47"/>
+      <c r="BM11" s="0"/>
+      <c r="BN11" s="0"/>
       <c r="BO11" s="47"/>
       <c r="BP11" s="47"/>
       <c r="BQ11" s="47"/>
@@ -21874,8 +21842,8 @@
       <c r="AR12" s="34"/>
       <c r="AS12" s="16"/>
       <c r="AT12" s="47"/>
-      <c r="AU12" s="47"/>
-      <c r="AV12" s="47"/>
+      <c r="AU12" s="0"/>
+      <c r="AV12" s="0"/>
       <c r="AW12" s="47"/>
       <c r="AX12" s="47"/>
       <c r="AY12" s="47"/>
@@ -21892,8 +21860,8 @@
       <c r="BJ12" s="47"/>
       <c r="BK12" s="47"/>
       <c r="BL12" s="47"/>
-      <c r="BM12" s="47"/>
-      <c r="BN12" s="47"/>
+      <c r="BM12" s="0"/>
+      <c r="BN12" s="0"/>
       <c r="BO12" s="47"/>
       <c r="BP12" s="47"/>
       <c r="BQ12" s="47"/>
@@ -21962,8 +21930,8 @@
       <c r="AR13" s="34"/>
       <c r="AS13" s="16"/>
       <c r="AT13" s="47"/>
-      <c r="AU13" s="47"/>
-      <c r="AV13" s="47"/>
+      <c r="AU13" s="0"/>
+      <c r="AV13" s="0"/>
       <c r="AW13" s="47"/>
       <c r="AX13" s="47"/>
       <c r="AY13" s="47"/>
@@ -21980,8 +21948,8 @@
       <c r="BJ13" s="47"/>
       <c r="BK13" s="47"/>
       <c r="BL13" s="47"/>
-      <c r="BM13" s="47"/>
-      <c r="BN13" s="47"/>
+      <c r="BM13" s="0"/>
+      <c r="BN13" s="0"/>
       <c r="BO13" s="47"/>
       <c r="BP13" s="47"/>
       <c r="BQ13" s="47"/>
@@ -22050,8 +22018,8 @@
       <c r="AR14" s="34"/>
       <c r="AS14" s="16"/>
       <c r="AT14" s="47"/>
-      <c r="AU14" s="47"/>
-      <c r="AV14" s="47"/>
+      <c r="AU14" s="0"/>
+      <c r="AV14" s="0"/>
       <c r="AW14" s="47"/>
       <c r="AX14" s="47"/>
       <c r="AY14" s="47"/>
@@ -22068,8 +22036,8 @@
       <c r="BJ14" s="47"/>
       <c r="BK14" s="47"/>
       <c r="BL14" s="47"/>
-      <c r="BM14" s="47"/>
-      <c r="BN14" s="47"/>
+      <c r="BM14" s="0"/>
+      <c r="BN14" s="0"/>
       <c r="BO14" s="47"/>
       <c r="BP14" s="47"/>
       <c r="BQ14" s="47"/>
@@ -22138,8 +22106,8 @@
       <c r="AR15" s="34"/>
       <c r="AS15" s="16"/>
       <c r="AT15" s="47"/>
-      <c r="AU15" s="47"/>
-      <c r="AV15" s="47"/>
+      <c r="AU15" s="0"/>
+      <c r="AV15" s="0"/>
       <c r="AW15" s="47"/>
       <c r="AX15" s="47"/>
       <c r="AY15" s="47"/>
@@ -22156,8 +22124,8 @@
       <c r="BJ15" s="47"/>
       <c r="BK15" s="47"/>
       <c r="BL15" s="47"/>
-      <c r="BM15" s="47"/>
-      <c r="BN15" s="47"/>
+      <c r="BM15" s="0"/>
+      <c r="BN15" s="0"/>
       <c r="BO15" s="47"/>
       <c r="BP15" s="47"/>
       <c r="BQ15" s="47"/>
@@ -22226,8 +22194,8 @@
       <c r="AR16" s="34"/>
       <c r="AS16" s="16"/>
       <c r="AT16" s="47"/>
-      <c r="AU16" s="47"/>
-      <c r="AV16" s="47"/>
+      <c r="AU16" s="0"/>
+      <c r="AV16" s="0"/>
       <c r="AW16" s="47"/>
       <c r="AX16" s="47"/>
       <c r="AY16" s="47"/>
@@ -22244,8 +22212,8 @@
       <c r="BJ16" s="47"/>
       <c r="BK16" s="47"/>
       <c r="BL16" s="47"/>
-      <c r="BM16" s="47"/>
-      <c r="BN16" s="47"/>
+      <c r="BM16" s="0"/>
+      <c r="BN16" s="0"/>
       <c r="BO16" s="47"/>
       <c r="BP16" s="47"/>
       <c r="BQ16" s="47"/>
@@ -22314,8 +22282,8 @@
       <c r="AR17" s="34"/>
       <c r="AS17" s="16"/>
       <c r="AT17" s="47"/>
-      <c r="AU17" s="47"/>
-      <c r="AV17" s="47"/>
+      <c r="AU17" s="0"/>
+      <c r="AV17" s="0"/>
       <c r="AW17" s="47"/>
       <c r="AX17" s="47"/>
       <c r="AY17" s="47"/>
@@ -22332,8 +22300,8 @@
       <c r="BJ17" s="47"/>
       <c r="BK17" s="47"/>
       <c r="BL17" s="47"/>
-      <c r="BM17" s="47"/>
-      <c r="BN17" s="47"/>
+      <c r="BM17" s="0"/>
+      <c r="BN17" s="0"/>
       <c r="BO17" s="47"/>
       <c r="BP17" s="47"/>
       <c r="BQ17" s="47"/>
@@ -22402,8 +22370,8 @@
       <c r="AR18" s="34"/>
       <c r="AS18" s="16"/>
       <c r="AT18" s="47"/>
-      <c r="AU18" s="47"/>
-      <c r="AV18" s="47"/>
+      <c r="AU18" s="0"/>
+      <c r="AV18" s="0"/>
       <c r="AW18" s="47"/>
       <c r="AX18" s="47"/>
       <c r="AY18" s="47"/>
@@ -22420,8 +22388,8 @@
       <c r="BJ18" s="47"/>
       <c r="BK18" s="47"/>
       <c r="BL18" s="47"/>
-      <c r="BM18" s="47"/>
-      <c r="BN18" s="47"/>
+      <c r="BM18" s="0"/>
+      <c r="BN18" s="0"/>
       <c r="BO18" s="47"/>
       <c r="BP18" s="47"/>
       <c r="BQ18" s="47"/>
@@ -22478,8 +22446,8 @@
       <c r="AR19" s="19"/>
       <c r="AS19" s="16"/>
       <c r="AT19" s="47"/>
-      <c r="AU19" s="47"/>
-      <c r="AV19" s="47"/>
+      <c r="AU19" s="0"/>
+      <c r="AV19" s="0"/>
       <c r="AW19" s="47"/>
       <c r="AX19" s="47"/>
       <c r="AY19" s="47"/>
@@ -22496,8 +22464,8 @@
       <c r="BJ19" s="47"/>
       <c r="BK19" s="47"/>
       <c r="BL19" s="47"/>
-      <c r="BM19" s="47"/>
-      <c r="BN19" s="47"/>
+      <c r="BM19" s="0"/>
+      <c r="BN19" s="0"/>
       <c r="BO19" s="47"/>
       <c r="BP19" s="47"/>
       <c r="BQ19" s="47"/>
@@ -22809,12 +22777,8 @@
       <c r="AT22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV22" s="49" t="s">
-        <v>90</v>
-      </c>
+      <c r="AU22" s="0"/>
+      <c r="AV22" s="0"/>
       <c r="AW22" s="49" t="s">
         <v>91</v>
       </c>
@@ -22863,12 +22827,8 @@
       <c r="BL22" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="BM22" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN22" s="49" t="s">
-        <v>108</v>
-      </c>
+      <c r="BM22" s="0"/>
+      <c r="BN22" s="0"/>
       <c r="BO22" s="49" t="s">
         <v>94</v>
       </c>
@@ -22898,14 +22858,14 @@
       <c r="F23" s="28">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>130</v>
       </c>
       <c r="H23" s="28">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>120</v>
       </c>
       <c r="J23" s="28">
@@ -23043,11 +23003,11 @@
       <c r="AT23" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="47" t="s">
+      <c r="AU23" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="AV23" s="47" t="s">
-        <v>140</v>
+      <c r="AV23" t="s" s="0">
+        <v>160</v>
       </c>
       <c r="AW23" s="50">
         <f>AM23</f>
@@ -23087,11 +23047,11 @@
       <c r="BL23" s="50" t="s">
         <v>119</v>
       </c>
-      <c r="BM23" s="47" t="s">
-        <v>140</v>
-      </c>
-      <c r="BN23" s="47" t="s">
-        <v>141</v>
+      <c r="BM23" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>165</v>
       </c>
       <c r="BO23" s="50">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Added production module test scenarios and updated PO test data sheets
Added production module test scenarios and updated PO test data sheets
</commit_message>
<xml_diff>
--- a/testdata/DirectGRN-FOC Scenarios.xlsx
+++ b/testdata/DirectGRN-FOC Scenarios.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="7" activeTab="8"/>
+    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="6" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="ImportDirectGRNUDGeneralSameUOM" sheetId="2" r:id="rId1"/>
@@ -355,7 +355,7 @@
     <t>Qty After Post forSource Warehouse</t>
   </si>
   <si>
-    <t>GWL_ITEM_SIMILAR-1</t>
+    <t>ITEM-GWL-SIMILAR-01</t>
   </si>
   <si>
     <t>HSN1</t>
@@ -415,7 +415,7 @@
     <t>Qty Before Post For Source WareHouse</t>
   </si>
   <si>
-    <t>GWL_SERVICE-ITEM_SIMILAR-1</t>
+    <t>ITEM-GWL-SERVICE-01</t>
   </si>
   <si>
     <t>INS WH-1</t>
@@ -439,7 +439,7 @@
     <t>Before Unit Cost</t>
   </si>
   <si>
-    <t>GWL_ITEM_SIMILAR-RC-1</t>
+    <t>ITEM-GWL-SIMILAR-RC-01</t>
   </si>
   <si>
     <t>8106.9762</t>
@@ -448,7 +448,7 @@
     <t>42</t>
   </si>
   <si>
-    <t>GWL_SERVICE-ITEM_SIMILAR-RC-1</t>
+    <t>ITEM-GWL-SERVICE-RC-01</t>
   </si>
   <si>
     <t>GWL_ITEM_SIMILAR-PL-1</t>
@@ -475,7 +475,7 @@
     <t>Unit Qunatity Before</t>
   </si>
   <si>
-    <t>GWL_ITEM_DISSIMILAR-1</t>
+    <t>ITEM-GWL-DISSIMILAR-01</t>
   </si>
   <si>
     <t>23750.7</t>
@@ -487,7 +487,7 @@
     <t>20.677</t>
   </si>
   <si>
-    <t>GWL_ITEM_DISSIMILAR-RC-1</t>
+    <t>ITEM-GWL-DISSIMILAR-RC-01</t>
   </si>
   <si>
     <t>24548.34001</t>
@@ -519,7 +519,7 @@
     <numFmt numFmtId="182" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="183" formatCode="0.00000_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -562,6 +562,11 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri Light"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1305,16 +1310,13 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1323,122 +1325,125 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1566,10 +1571,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1593,7 +1599,7 @@
     <xf numFmtId="180" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="183" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1605,7 +1611,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2064,102 +2070,102 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.5" spans="1:45">
-      <c r="A1" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="70"/>
-      <c r="W1" s="70"/>
-      <c r="X1" s="70"/>
-      <c r="Y1" s="70"/>
-      <c r="Z1" s="70"/>
-      <c r="AA1" s="70"/>
-      <c r="AB1" s="70"/>
-      <c r="AC1" s="70"/>
-      <c r="AD1" s="70"/>
-      <c r="AE1" s="70"/>
-      <c r="AF1" s="70"/>
-      <c r="AG1" s="70"/>
-      <c r="AH1" s="70"/>
-      <c r="AI1" s="70"/>
-      <c r="AJ1" s="70"/>
-      <c r="AK1" s="70"/>
-      <c r="AL1" s="70"/>
-      <c r="AM1" s="70"/>
-      <c r="AN1" s="70"/>
-      <c r="AO1" s="70"/>
-      <c r="AP1" s="70"/>
-      <c r="AQ1" s="70"/>
-      <c r="AR1" s="71"/>
-      <c r="AS1" s="71"/>
+      <c r="A1" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
+      <c r="W1" s="71"/>
+      <c r="X1" s="71"/>
+      <c r="Y1" s="71"/>
+      <c r="Z1" s="71"/>
+      <c r="AA1" s="71"/>
+      <c r="AB1" s="71"/>
+      <c r="AC1" s="71"/>
+      <c r="AD1" s="71"/>
+      <c r="AE1" s="71"/>
+      <c r="AF1" s="71"/>
+      <c r="AG1" s="71"/>
+      <c r="AH1" s="71"/>
+      <c r="AI1" s="71"/>
+      <c r="AJ1" s="71"/>
+      <c r="AK1" s="71"/>
+      <c r="AL1" s="71"/>
+      <c r="AM1" s="71"/>
+      <c r="AN1" s="71"/>
+      <c r="AO1" s="71"/>
+      <c r="AP1" s="71"/>
+      <c r="AQ1" s="71"/>
+      <c r="AR1" s="72"/>
+      <c r="AS1" s="72"/>
     </row>
     <row r="2" ht="19.25" spans="1:45">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="T2" s="70"/>
-      <c r="U2" s="70"/>
-      <c r="V2" s="70"/>
-      <c r="W2" s="70"/>
-      <c r="X2" s="70"/>
-      <c r="Y2" s="70"/>
-      <c r="Z2" s="70"/>
-      <c r="AA2" s="70"/>
-      <c r="AB2" s="70"/>
-      <c r="AC2" s="70"/>
-      <c r="AD2" s="70"/>
-      <c r="AE2" s="70"/>
-      <c r="AF2" s="70"/>
-      <c r="AG2" s="70"/>
-      <c r="AH2" s="70"/>
-      <c r="AI2" s="70"/>
-      <c r="AJ2" s="70"/>
-      <c r="AK2" s="70"/>
-      <c r="AL2" s="70"/>
-      <c r="AM2" s="70"/>
-      <c r="AN2" s="70"/>
-      <c r="AO2" s="70"/>
-      <c r="AP2" s="70"/>
-      <c r="AQ2" s="70"/>
-      <c r="AR2" s="71"/>
-      <c r="AS2" s="71"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="71"/>
+      <c r="Q2" s="71"/>
+      <c r="R2" s="71"/>
+      <c r="S2" s="71"/>
+      <c r="T2" s="71"/>
+      <c r="U2" s="71"/>
+      <c r="V2" s="71"/>
+      <c r="W2" s="71"/>
+      <c r="X2" s="71"/>
+      <c r="Y2" s="71"/>
+      <c r="Z2" s="71"/>
+      <c r="AA2" s="71"/>
+      <c r="AB2" s="71"/>
+      <c r="AC2" s="71"/>
+      <c r="AD2" s="71"/>
+      <c r="AE2" s="71"/>
+      <c r="AF2" s="71"/>
+      <c r="AG2" s="71"/>
+      <c r="AH2" s="71"/>
+      <c r="AI2" s="71"/>
+      <c r="AJ2" s="71"/>
+      <c r="AK2" s="71"/>
+      <c r="AL2" s="71"/>
+      <c r="AM2" s="71"/>
+      <c r="AN2" s="71"/>
+      <c r="AO2" s="71"/>
+      <c r="AP2" s="71"/>
+      <c r="AQ2" s="71"/>
+      <c r="AR2" s="72"/>
+      <c r="AS2" s="72"/>
     </row>
     <row r="3" ht="15.25" spans="1:45">
       <c r="A3" s="5" t="s">
@@ -2222,970 +2228,970 @@
       <c r="AP3" s="9"/>
       <c r="AQ3" s="9"/>
       <c r="AR3" s="9"/>
-      <c r="AS3" s="71"/>
+      <c r="AS3" s="72"/>
     </row>
     <row r="4" spans="1:45">
-      <c r="A4" s="72">
+      <c r="A4" s="73">
         <v>1</v>
       </c>
-      <c r="B4" s="73" t="s">
+      <c r="B4" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="73" t="s">
+      <c r="C4" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="74">
+      <c r="D4" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="75">
         <v>25</v>
       </c>
-      <c r="G4" s="75">
+      <c r="G4" s="76">
         <v>257.63</v>
       </c>
-      <c r="H4" s="76">
+      <c r="H4" s="77">
         <f t="shared" ref="H4:H18" si="0">F4*G4</f>
         <v>6440.75</v>
       </c>
-      <c r="I4" s="77"/>
-      <c r="J4" s="77"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="78"/>
-      <c r="N4" s="78"/>
-      <c r="O4" s="78"/>
-      <c r="P4" s="78"/>
-      <c r="Q4" s="78"/>
-      <c r="R4" s="78"/>
-      <c r="S4" s="78"/>
-      <c r="T4" s="78"/>
-      <c r="U4" s="77"/>
-      <c r="V4" s="77"/>
-      <c r="W4" s="77"/>
-      <c r="X4" s="77"/>
-      <c r="Y4" s="77"/>
-      <c r="Z4" s="77"/>
-      <c r="AA4" s="77"/>
-      <c r="AB4" s="78"/>
-      <c r="AC4" s="78"/>
-      <c r="AD4" s="78"/>
-      <c r="AE4" s="78"/>
-      <c r="AF4" s="78"/>
-      <c r="AG4" s="78"/>
-      <c r="AH4" s="78"/>
-      <c r="AI4" s="78"/>
-      <c r="AJ4" s="78"/>
-      <c r="AK4" s="78"/>
-      <c r="AL4" s="78"/>
-      <c r="AM4" s="78"/>
-      <c r="AN4" s="78"/>
-      <c r="AO4" s="78"/>
-      <c r="AP4" s="78"/>
-      <c r="AQ4" s="78"/>
-      <c r="AR4" s="78"/>
-      <c r="AS4" s="71"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
+      <c r="N4" s="79"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="79"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="78"/>
+      <c r="V4" s="78"/>
+      <c r="W4" s="78"/>
+      <c r="X4" s="78"/>
+      <c r="Y4" s="78"/>
+      <c r="Z4" s="78"/>
+      <c r="AA4" s="78"/>
+      <c r="AB4" s="79"/>
+      <c r="AC4" s="79"/>
+      <c r="AD4" s="79"/>
+      <c r="AE4" s="79"/>
+      <c r="AF4" s="79"/>
+      <c r="AG4" s="79"/>
+      <c r="AH4" s="79"/>
+      <c r="AI4" s="79"/>
+      <c r="AJ4" s="79"/>
+      <c r="AK4" s="79"/>
+      <c r="AL4" s="79"/>
+      <c r="AM4" s="79"/>
+      <c r="AN4" s="79"/>
+      <c r="AO4" s="79"/>
+      <c r="AP4" s="79"/>
+      <c r="AQ4" s="79"/>
+      <c r="AR4" s="79"/>
+      <c r="AS4" s="72"/>
     </row>
     <row r="5" spans="1:45">
-      <c r="A5" s="72">
+      <c r="A5" s="73">
         <v>2</v>
       </c>
-      <c r="B5" s="73" t="s">
+      <c r="B5" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="73" t="s">
+      <c r="C5" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="74">
+      <c r="D5" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="75">
         <v>35</v>
       </c>
-      <c r="G5" s="75">
+      <c r="G5" s="76">
         <v>125.45</v>
       </c>
-      <c r="H5" s="76">
+      <c r="H5" s="77">
         <f t="shared" si="0"/>
         <v>4390.75</v>
       </c>
-      <c r="I5" s="77"/>
-      <c r="J5" s="77"/>
-      <c r="K5" s="77"/>
-      <c r="L5" s="78"/>
-      <c r="M5" s="78"/>
-      <c r="N5" s="78"/>
-      <c r="O5" s="78"/>
-      <c r="P5" s="78"/>
-      <c r="Q5" s="78"/>
-      <c r="R5" s="78"/>
-      <c r="S5" s="78"/>
-      <c r="T5" s="78"/>
-      <c r="U5" s="77"/>
-      <c r="V5" s="77"/>
-      <c r="W5" s="77"/>
-      <c r="X5" s="77"/>
-      <c r="Y5" s="77"/>
-      <c r="Z5" s="77"/>
-      <c r="AA5" s="77"/>
-      <c r="AB5" s="78"/>
-      <c r="AC5" s="78"/>
-      <c r="AD5" s="78"/>
-      <c r="AE5" s="78"/>
-      <c r="AF5" s="78"/>
-      <c r="AG5" s="78"/>
-      <c r="AH5" s="78"/>
-      <c r="AI5" s="78"/>
-      <c r="AJ5" s="78"/>
-      <c r="AK5" s="78"/>
-      <c r="AL5" s="78"/>
-      <c r="AM5" s="78"/>
-      <c r="AN5" s="78"/>
-      <c r="AO5" s="78"/>
-      <c r="AP5" s="78"/>
-      <c r="AQ5" s="78"/>
-      <c r="AR5" s="78"/>
-      <c r="AS5" s="71"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="78"/>
+      <c r="K5" s="78"/>
+      <c r="L5" s="79"/>
+      <c r="M5" s="79"/>
+      <c r="N5" s="79"/>
+      <c r="O5" s="79"/>
+      <c r="P5" s="79"/>
+      <c r="Q5" s="79"/>
+      <c r="R5" s="79"/>
+      <c r="S5" s="79"/>
+      <c r="T5" s="79"/>
+      <c r="U5" s="78"/>
+      <c r="V5" s="78"/>
+      <c r="W5" s="78"/>
+      <c r="X5" s="78"/>
+      <c r="Y5" s="78"/>
+      <c r="Z5" s="78"/>
+      <c r="AA5" s="78"/>
+      <c r="AB5" s="79"/>
+      <c r="AC5" s="79"/>
+      <c r="AD5" s="79"/>
+      <c r="AE5" s="79"/>
+      <c r="AF5" s="79"/>
+      <c r="AG5" s="79"/>
+      <c r="AH5" s="79"/>
+      <c r="AI5" s="79"/>
+      <c r="AJ5" s="79"/>
+      <c r="AK5" s="79"/>
+      <c r="AL5" s="79"/>
+      <c r="AM5" s="79"/>
+      <c r="AN5" s="79"/>
+      <c r="AO5" s="79"/>
+      <c r="AP5" s="79"/>
+      <c r="AQ5" s="79"/>
+      <c r="AR5" s="79"/>
+      <c r="AS5" s="72"/>
     </row>
     <row r="6" spans="1:45">
-      <c r="A6" s="72">
+      <c r="A6" s="73">
         <v>3</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="B6" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="73" t="s">
+      <c r="C6" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="74">
+      <c r="D6" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="75">
         <v>45</v>
       </c>
-      <c r="G6" s="75">
+      <c r="G6" s="76">
         <v>125.36</v>
       </c>
-      <c r="H6" s="76">
+      <c r="H6" s="77">
         <f t="shared" si="0"/>
         <v>5641.2</v>
       </c>
-      <c r="I6" s="77"/>
-      <c r="J6" s="77"/>
-      <c r="K6" s="77"/>
-      <c r="L6" s="78"/>
-      <c r="M6" s="78"/>
-      <c r="N6" s="78"/>
-      <c r="O6" s="78"/>
-      <c r="P6" s="78"/>
-      <c r="Q6" s="78"/>
-      <c r="R6" s="78"/>
-      <c r="S6" s="78"/>
-      <c r="T6" s="78"/>
-      <c r="U6" s="77"/>
-      <c r="V6" s="77"/>
-      <c r="W6" s="77"/>
-      <c r="X6" s="77"/>
-      <c r="Y6" s="77"/>
-      <c r="Z6" s="77"/>
-      <c r="AA6" s="77"/>
-      <c r="AB6" s="78"/>
-      <c r="AC6" s="78"/>
-      <c r="AD6" s="78"/>
-      <c r="AE6" s="78"/>
-      <c r="AF6" s="78"/>
-      <c r="AG6" s="78"/>
-      <c r="AH6" s="78"/>
-      <c r="AI6" s="78"/>
-      <c r="AJ6" s="78"/>
-      <c r="AK6" s="78"/>
-      <c r="AL6" s="78"/>
-      <c r="AM6" s="78"/>
-      <c r="AN6" s="78"/>
-      <c r="AO6" s="78"/>
-      <c r="AP6" s="78"/>
-      <c r="AQ6" s="78"/>
-      <c r="AR6" s="78"/>
-      <c r="AS6" s="71"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="78"/>
+      <c r="K6" s="78"/>
+      <c r="L6" s="79"/>
+      <c r="M6" s="79"/>
+      <c r="N6" s="79"/>
+      <c r="O6" s="79"/>
+      <c r="P6" s="79"/>
+      <c r="Q6" s="79"/>
+      <c r="R6" s="79"/>
+      <c r="S6" s="79"/>
+      <c r="T6" s="79"/>
+      <c r="U6" s="78"/>
+      <c r="V6" s="78"/>
+      <c r="W6" s="78"/>
+      <c r="X6" s="78"/>
+      <c r="Y6" s="78"/>
+      <c r="Z6" s="78"/>
+      <c r="AA6" s="78"/>
+      <c r="AB6" s="79"/>
+      <c r="AC6" s="79"/>
+      <c r="AD6" s="79"/>
+      <c r="AE6" s="79"/>
+      <c r="AF6" s="79"/>
+      <c r="AG6" s="79"/>
+      <c r="AH6" s="79"/>
+      <c r="AI6" s="79"/>
+      <c r="AJ6" s="79"/>
+      <c r="AK6" s="79"/>
+      <c r="AL6" s="79"/>
+      <c r="AM6" s="79"/>
+      <c r="AN6" s="79"/>
+      <c r="AO6" s="79"/>
+      <c r="AP6" s="79"/>
+      <c r="AQ6" s="79"/>
+      <c r="AR6" s="79"/>
+      <c r="AS6" s="72"/>
     </row>
     <row r="7" spans="1:45">
-      <c r="A7" s="72">
+      <c r="A7" s="73">
         <v>4</v>
       </c>
-      <c r="B7" s="73" t="s">
+      <c r="B7" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="73" t="s">
+      <c r="C7" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="74">
+      <c r="D7" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="75">
         <v>55</v>
       </c>
-      <c r="G7" s="75">
+      <c r="G7" s="76">
         <v>45.25</v>
       </c>
-      <c r="H7" s="76">
+      <c r="H7" s="77">
         <f t="shared" si="0"/>
         <v>2488.75</v>
       </c>
-      <c r="I7" s="77"/>
-      <c r="J7" s="77"/>
-      <c r="K7" s="77"/>
-      <c r="L7" s="78"/>
-      <c r="M7" s="78"/>
-      <c r="N7" s="78"/>
-      <c r="O7" s="78"/>
-      <c r="P7" s="78"/>
-      <c r="Q7" s="78"/>
-      <c r="R7" s="78"/>
-      <c r="S7" s="78"/>
-      <c r="T7" s="78"/>
-      <c r="U7" s="77"/>
-      <c r="V7" s="77"/>
-      <c r="W7" s="77"/>
-      <c r="X7" s="77"/>
-      <c r="Y7" s="77"/>
-      <c r="Z7" s="77"/>
-      <c r="AA7" s="77"/>
-      <c r="AB7" s="78"/>
-      <c r="AC7" s="78"/>
-      <c r="AD7" s="78"/>
-      <c r="AE7" s="78"/>
-      <c r="AF7" s="78"/>
-      <c r="AG7" s="78"/>
-      <c r="AH7" s="78"/>
-      <c r="AI7" s="78"/>
-      <c r="AJ7" s="78"/>
-      <c r="AK7" s="78"/>
-      <c r="AL7" s="78"/>
-      <c r="AM7" s="78"/>
-      <c r="AN7" s="78"/>
-      <c r="AO7" s="78"/>
-      <c r="AP7" s="78"/>
-      <c r="AQ7" s="78"/>
-      <c r="AR7" s="78"/>
-      <c r="AS7" s="71"/>
+      <c r="I7" s="78"/>
+      <c r="J7" s="78"/>
+      <c r="K7" s="78"/>
+      <c r="L7" s="79"/>
+      <c r="M7" s="79"/>
+      <c r="N7" s="79"/>
+      <c r="O7" s="79"/>
+      <c r="P7" s="79"/>
+      <c r="Q7" s="79"/>
+      <c r="R7" s="79"/>
+      <c r="S7" s="79"/>
+      <c r="T7" s="79"/>
+      <c r="U7" s="78"/>
+      <c r="V7" s="78"/>
+      <c r="W7" s="78"/>
+      <c r="X7" s="78"/>
+      <c r="Y7" s="78"/>
+      <c r="Z7" s="78"/>
+      <c r="AA7" s="78"/>
+      <c r="AB7" s="79"/>
+      <c r="AC7" s="79"/>
+      <c r="AD7" s="79"/>
+      <c r="AE7" s="79"/>
+      <c r="AF7" s="79"/>
+      <c r="AG7" s="79"/>
+      <c r="AH7" s="79"/>
+      <c r="AI7" s="79"/>
+      <c r="AJ7" s="79"/>
+      <c r="AK7" s="79"/>
+      <c r="AL7" s="79"/>
+      <c r="AM7" s="79"/>
+      <c r="AN7" s="79"/>
+      <c r="AO7" s="79"/>
+      <c r="AP7" s="79"/>
+      <c r="AQ7" s="79"/>
+      <c r="AR7" s="79"/>
+      <c r="AS7" s="72"/>
     </row>
     <row r="8" spans="1:45">
-      <c r="A8" s="72">
+      <c r="A8" s="73">
         <v>5</v>
       </c>
-      <c r="B8" s="73" t="s">
+      <c r="B8" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="73" t="s">
+      <c r="C8" s="74" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="74">
+      <c r="D8" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="75">
         <v>60</v>
       </c>
-      <c r="G8" s="75">
+      <c r="G8" s="76">
         <v>45.5</v>
       </c>
-      <c r="H8" s="76">
+      <c r="H8" s="77">
         <f t="shared" si="0"/>
         <v>2730</v>
       </c>
-      <c r="I8" s="77"/>
-      <c r="J8" s="77"/>
-      <c r="K8" s="77"/>
-      <c r="L8" s="78"/>
-      <c r="M8" s="78"/>
-      <c r="N8" s="78"/>
-      <c r="O8" s="78"/>
-      <c r="P8" s="78"/>
-      <c r="Q8" s="78"/>
-      <c r="R8" s="78"/>
-      <c r="S8" s="78"/>
-      <c r="T8" s="78"/>
-      <c r="U8" s="77"/>
-      <c r="V8" s="77"/>
-      <c r="W8" s="77"/>
-      <c r="X8" s="77"/>
-      <c r="Y8" s="77"/>
-      <c r="Z8" s="77"/>
-      <c r="AA8" s="77"/>
-      <c r="AB8" s="78"/>
-      <c r="AC8" s="78"/>
-      <c r="AD8" s="78"/>
-      <c r="AE8" s="78"/>
-      <c r="AF8" s="78"/>
-      <c r="AG8" s="78"/>
-      <c r="AH8" s="78"/>
-      <c r="AI8" s="78"/>
-      <c r="AJ8" s="78"/>
-      <c r="AK8" s="78"/>
-      <c r="AL8" s="78"/>
-      <c r="AM8" s="78"/>
-      <c r="AN8" s="78"/>
-      <c r="AO8" s="78"/>
-      <c r="AP8" s="78"/>
-      <c r="AQ8" s="78"/>
-      <c r="AR8" s="78"/>
-      <c r="AS8" s="71"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="78"/>
+      <c r="K8" s="78"/>
+      <c r="L8" s="79"/>
+      <c r="M8" s="79"/>
+      <c r="N8" s="79"/>
+      <c r="O8" s="79"/>
+      <c r="P8" s="79"/>
+      <c r="Q8" s="79"/>
+      <c r="R8" s="79"/>
+      <c r="S8" s="79"/>
+      <c r="T8" s="79"/>
+      <c r="U8" s="78"/>
+      <c r="V8" s="78"/>
+      <c r="W8" s="78"/>
+      <c r="X8" s="78"/>
+      <c r="Y8" s="78"/>
+      <c r="Z8" s="78"/>
+      <c r="AA8" s="78"/>
+      <c r="AB8" s="79"/>
+      <c r="AC8" s="79"/>
+      <c r="AD8" s="79"/>
+      <c r="AE8" s="79"/>
+      <c r="AF8" s="79"/>
+      <c r="AG8" s="79"/>
+      <c r="AH8" s="79"/>
+      <c r="AI8" s="79"/>
+      <c r="AJ8" s="79"/>
+      <c r="AK8" s="79"/>
+      <c r="AL8" s="79"/>
+      <c r="AM8" s="79"/>
+      <c r="AN8" s="79"/>
+      <c r="AO8" s="79"/>
+      <c r="AP8" s="79"/>
+      <c r="AQ8" s="79"/>
+      <c r="AR8" s="79"/>
+      <c r="AS8" s="72"/>
     </row>
     <row r="9" spans="1:45">
-      <c r="A9" s="72">
+      <c r="A9" s="73">
         <v>6</v>
       </c>
-      <c r="B9" s="73" t="s">
+      <c r="B9" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="73" t="s">
+      <c r="C9" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="74">
+      <c r="D9" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="75">
         <v>75</v>
       </c>
-      <c r="G9" s="75">
+      <c r="G9" s="76">
         <v>125.25</v>
       </c>
-      <c r="H9" s="76">
+      <c r="H9" s="77">
         <f t="shared" si="0"/>
         <v>9393.75</v>
       </c>
-      <c r="I9" s="77"/>
-      <c r="J9" s="77"/>
-      <c r="K9" s="77"/>
-      <c r="L9" s="78"/>
-      <c r="M9" s="78"/>
-      <c r="N9" s="78"/>
-      <c r="O9" s="78"/>
-      <c r="P9" s="78"/>
-      <c r="Q9" s="78"/>
-      <c r="R9" s="78"/>
-      <c r="S9" s="78"/>
-      <c r="T9" s="78"/>
-      <c r="U9" s="77"/>
-      <c r="V9" s="77"/>
-      <c r="W9" s="77"/>
-      <c r="X9" s="77"/>
-      <c r="Y9" s="77"/>
-      <c r="Z9" s="77"/>
-      <c r="AA9" s="77"/>
-      <c r="AB9" s="78"/>
-      <c r="AC9" s="78"/>
-      <c r="AD9" s="78"/>
-      <c r="AE9" s="78"/>
-      <c r="AF9" s="78"/>
-      <c r="AG9" s="78"/>
-      <c r="AH9" s="78"/>
-      <c r="AI9" s="78"/>
-      <c r="AJ9" s="78"/>
-      <c r="AK9" s="78"/>
-      <c r="AL9" s="78"/>
-      <c r="AM9" s="78"/>
-      <c r="AN9" s="78"/>
-      <c r="AO9" s="78"/>
-      <c r="AP9" s="78"/>
-      <c r="AQ9" s="78"/>
-      <c r="AR9" s="78"/>
-      <c r="AS9" s="71"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="78"/>
+      <c r="K9" s="78"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+      <c r="N9" s="79"/>
+      <c r="O9" s="79"/>
+      <c r="P9" s="79"/>
+      <c r="Q9" s="79"/>
+      <c r="R9" s="79"/>
+      <c r="S9" s="79"/>
+      <c r="T9" s="79"/>
+      <c r="U9" s="78"/>
+      <c r="V9" s="78"/>
+      <c r="W9" s="78"/>
+      <c r="X9" s="78"/>
+      <c r="Y9" s="78"/>
+      <c r="Z9" s="78"/>
+      <c r="AA9" s="78"/>
+      <c r="AB9" s="79"/>
+      <c r="AC9" s="79"/>
+      <c r="AD9" s="79"/>
+      <c r="AE9" s="79"/>
+      <c r="AF9" s="79"/>
+      <c r="AG9" s="79"/>
+      <c r="AH9" s="79"/>
+      <c r="AI9" s="79"/>
+      <c r="AJ9" s="79"/>
+      <c r="AK9" s="79"/>
+      <c r="AL9" s="79"/>
+      <c r="AM9" s="79"/>
+      <c r="AN9" s="79"/>
+      <c r="AO9" s="79"/>
+      <c r="AP9" s="79"/>
+      <c r="AQ9" s="79"/>
+      <c r="AR9" s="79"/>
+      <c r="AS9" s="72"/>
     </row>
     <row r="10" spans="1:45">
-      <c r="A10" s="72">
+      <c r="A10" s="73">
         <v>7</v>
       </c>
-      <c r="B10" s="73" t="s">
+      <c r="B10" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="73" t="s">
+      <c r="C10" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="74">
+      <c r="D10" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="75">
         <v>28</v>
       </c>
-      <c r="G10" s="75">
+      <c r="G10" s="76">
         <v>150.5</v>
       </c>
-      <c r="H10" s="76">
+      <c r="H10" s="77">
         <f t="shared" si="0"/>
         <v>4214</v>
       </c>
-      <c r="I10" s="77"/>
-      <c r="J10" s="77"/>
-      <c r="K10" s="77"/>
-      <c r="L10" s="78"/>
-      <c r="M10" s="78"/>
-      <c r="N10" s="78"/>
-      <c r="O10" s="78"/>
-      <c r="P10" s="78"/>
-      <c r="Q10" s="78"/>
-      <c r="R10" s="78"/>
-      <c r="S10" s="78"/>
-      <c r="T10" s="78"/>
-      <c r="U10" s="77"/>
-      <c r="V10" s="77"/>
-      <c r="W10" s="77"/>
-      <c r="X10" s="77"/>
-      <c r="Y10" s="77"/>
-      <c r="Z10" s="77"/>
-      <c r="AA10" s="77"/>
-      <c r="AB10" s="78"/>
-      <c r="AC10" s="78"/>
-      <c r="AD10" s="78"/>
-      <c r="AE10" s="78"/>
-      <c r="AF10" s="78"/>
-      <c r="AG10" s="78"/>
-      <c r="AH10" s="78"/>
-      <c r="AI10" s="78"/>
-      <c r="AJ10" s="78"/>
-      <c r="AK10" s="78"/>
-      <c r="AL10" s="78"/>
-      <c r="AM10" s="78"/>
-      <c r="AN10" s="78"/>
-      <c r="AO10" s="78"/>
-      <c r="AP10" s="78"/>
-      <c r="AQ10" s="78"/>
-      <c r="AR10" s="78"/>
-      <c r="AS10" s="71"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="78"/>
+      <c r="L10" s="79"/>
+      <c r="M10" s="79"/>
+      <c r="N10" s="79"/>
+      <c r="O10" s="79"/>
+      <c r="P10" s="79"/>
+      <c r="Q10" s="79"/>
+      <c r="R10" s="79"/>
+      <c r="S10" s="79"/>
+      <c r="T10" s="79"/>
+      <c r="U10" s="78"/>
+      <c r="V10" s="78"/>
+      <c r="W10" s="78"/>
+      <c r="X10" s="78"/>
+      <c r="Y10" s="78"/>
+      <c r="Z10" s="78"/>
+      <c r="AA10" s="78"/>
+      <c r="AB10" s="79"/>
+      <c r="AC10" s="79"/>
+      <c r="AD10" s="79"/>
+      <c r="AE10" s="79"/>
+      <c r="AF10" s="79"/>
+      <c r="AG10" s="79"/>
+      <c r="AH10" s="79"/>
+      <c r="AI10" s="79"/>
+      <c r="AJ10" s="79"/>
+      <c r="AK10" s="79"/>
+      <c r="AL10" s="79"/>
+      <c r="AM10" s="79"/>
+      <c r="AN10" s="79"/>
+      <c r="AO10" s="79"/>
+      <c r="AP10" s="79"/>
+      <c r="AQ10" s="79"/>
+      <c r="AR10" s="79"/>
+      <c r="AS10" s="72"/>
     </row>
     <row r="11" spans="1:45">
-      <c r="A11" s="72">
+      <c r="A11" s="73">
         <v>8</v>
       </c>
-      <c r="B11" s="73" t="s">
+      <c r="B11" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="73" t="s">
+      <c r="C11" s="74" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="74">
+      <c r="D11" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="75">
         <v>30</v>
       </c>
-      <c r="G11" s="75">
+      <c r="G11" s="76">
         <v>65.32</v>
       </c>
-      <c r="H11" s="76">
+      <c r="H11" s="77">
         <f t="shared" si="0"/>
         <v>1959.6</v>
       </c>
-      <c r="I11" s="77"/>
-      <c r="J11" s="77"/>
-      <c r="K11" s="77"/>
-      <c r="L11" s="78"/>
-      <c r="M11" s="78"/>
-      <c r="N11" s="78"/>
-      <c r="O11" s="78"/>
-      <c r="P11" s="78"/>
-      <c r="Q11" s="78"/>
-      <c r="R11" s="78"/>
-      <c r="S11" s="78"/>
-      <c r="T11" s="78"/>
-      <c r="U11" s="77"/>
-      <c r="V11" s="77"/>
-      <c r="W11" s="77"/>
-      <c r="X11" s="77"/>
-      <c r="Y11" s="77"/>
-      <c r="Z11" s="77"/>
-      <c r="AA11" s="77"/>
-      <c r="AB11" s="78"/>
-      <c r="AC11" s="78"/>
-      <c r="AD11" s="78"/>
-      <c r="AE11" s="78"/>
-      <c r="AF11" s="78"/>
-      <c r="AG11" s="78"/>
-      <c r="AH11" s="78"/>
-      <c r="AI11" s="78"/>
-      <c r="AJ11" s="78"/>
-      <c r="AK11" s="78"/>
-      <c r="AL11" s="78"/>
-      <c r="AM11" s="78"/>
-      <c r="AN11" s="78"/>
-      <c r="AO11" s="78"/>
-      <c r="AP11" s="78"/>
-      <c r="AQ11" s="78"/>
-      <c r="AR11" s="78"/>
-      <c r="AS11" s="71"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="78"/>
+      <c r="L11" s="79"/>
+      <c r="M11" s="79"/>
+      <c r="N11" s="79"/>
+      <c r="O11" s="79"/>
+      <c r="P11" s="79"/>
+      <c r="Q11" s="79"/>
+      <c r="R11" s="79"/>
+      <c r="S11" s="79"/>
+      <c r="T11" s="79"/>
+      <c r="U11" s="78"/>
+      <c r="V11" s="78"/>
+      <c r="W11" s="78"/>
+      <c r="X11" s="78"/>
+      <c r="Y11" s="78"/>
+      <c r="Z11" s="78"/>
+      <c r="AA11" s="78"/>
+      <c r="AB11" s="79"/>
+      <c r="AC11" s="79"/>
+      <c r="AD11" s="79"/>
+      <c r="AE11" s="79"/>
+      <c r="AF11" s="79"/>
+      <c r="AG11" s="79"/>
+      <c r="AH11" s="79"/>
+      <c r="AI11" s="79"/>
+      <c r="AJ11" s="79"/>
+      <c r="AK11" s="79"/>
+      <c r="AL11" s="79"/>
+      <c r="AM11" s="79"/>
+      <c r="AN11" s="79"/>
+      <c r="AO11" s="79"/>
+      <c r="AP11" s="79"/>
+      <c r="AQ11" s="79"/>
+      <c r="AR11" s="79"/>
+      <c r="AS11" s="72"/>
     </row>
     <row r="12" spans="1:45">
-      <c r="A12" s="72">
+      <c r="A12" s="73">
         <v>9</v>
       </c>
-      <c r="B12" s="73" t="s">
+      <c r="B12" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="73" t="s">
+      <c r="C12" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="74">
+      <c r="D12" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="75">
         <v>25</v>
       </c>
-      <c r="G12" s="75">
+      <c r="G12" s="76">
         <v>74.89</v>
       </c>
-      <c r="H12" s="76">
+      <c r="H12" s="77">
         <f t="shared" si="0"/>
         <v>1872.25</v>
       </c>
-      <c r="I12" s="77"/>
-      <c r="J12" s="77"/>
-      <c r="K12" s="77"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="78"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="78"/>
-      <c r="P12" s="78"/>
-      <c r="Q12" s="78"/>
-      <c r="R12" s="78"/>
-      <c r="S12" s="78"/>
-      <c r="T12" s="78"/>
-      <c r="U12" s="77"/>
-      <c r="V12" s="77"/>
-      <c r="W12" s="77"/>
-      <c r="X12" s="77"/>
-      <c r="Y12" s="77"/>
-      <c r="Z12" s="77"/>
-      <c r="AA12" s="77"/>
-      <c r="AB12" s="78"/>
-      <c r="AC12" s="78"/>
-      <c r="AD12" s="78"/>
-      <c r="AE12" s="78"/>
-      <c r="AF12" s="78"/>
-      <c r="AG12" s="78"/>
-      <c r="AH12" s="78"/>
-      <c r="AI12" s="78"/>
-      <c r="AJ12" s="78"/>
-      <c r="AK12" s="78"/>
-      <c r="AL12" s="78"/>
-      <c r="AM12" s="78"/>
-      <c r="AN12" s="78"/>
-      <c r="AO12" s="78"/>
-      <c r="AP12" s="78"/>
-      <c r="AQ12" s="78"/>
-      <c r="AR12" s="78"/>
-      <c r="AS12" s="71"/>
+      <c r="I12" s="78"/>
+      <c r="J12" s="78"/>
+      <c r="K12" s="78"/>
+      <c r="L12" s="79"/>
+      <c r="M12" s="79"/>
+      <c r="N12" s="79"/>
+      <c r="O12" s="79"/>
+      <c r="P12" s="79"/>
+      <c r="Q12" s="79"/>
+      <c r="R12" s="79"/>
+      <c r="S12" s="79"/>
+      <c r="T12" s="79"/>
+      <c r="U12" s="78"/>
+      <c r="V12" s="78"/>
+      <c r="W12" s="78"/>
+      <c r="X12" s="78"/>
+      <c r="Y12" s="78"/>
+      <c r="Z12" s="78"/>
+      <c r="AA12" s="78"/>
+      <c r="AB12" s="79"/>
+      <c r="AC12" s="79"/>
+      <c r="AD12" s="79"/>
+      <c r="AE12" s="79"/>
+      <c r="AF12" s="79"/>
+      <c r="AG12" s="79"/>
+      <c r="AH12" s="79"/>
+      <c r="AI12" s="79"/>
+      <c r="AJ12" s="79"/>
+      <c r="AK12" s="79"/>
+      <c r="AL12" s="79"/>
+      <c r="AM12" s="79"/>
+      <c r="AN12" s="79"/>
+      <c r="AO12" s="79"/>
+      <c r="AP12" s="79"/>
+      <c r="AQ12" s="79"/>
+      <c r="AR12" s="79"/>
+      <c r="AS12" s="72"/>
     </row>
     <row r="13" spans="1:45">
-      <c r="A13" s="72">
+      <c r="A13" s="73">
         <v>10</v>
       </c>
-      <c r="B13" s="73" t="s">
+      <c r="B13" s="74" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="73" t="s">
+      <c r="C13" s="74" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="74">
+      <c r="D13" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="75">
         <v>28</v>
       </c>
-      <c r="G13" s="75">
+      <c r="G13" s="76">
         <v>89.56</v>
       </c>
-      <c r="H13" s="76">
+      <c r="H13" s="77">
         <f t="shared" si="0"/>
         <v>2507.68</v>
       </c>
-      <c r="I13" s="77"/>
-      <c r="J13" s="77"/>
-      <c r="K13" s="77"/>
-      <c r="L13" s="78"/>
-      <c r="M13" s="78"/>
-      <c r="N13" s="78"/>
-      <c r="O13" s="78"/>
-      <c r="P13" s="78"/>
-      <c r="Q13" s="78"/>
-      <c r="R13" s="78"/>
-      <c r="S13" s="78"/>
-      <c r="T13" s="78"/>
-      <c r="U13" s="77"/>
-      <c r="V13" s="77"/>
-      <c r="W13" s="77"/>
-      <c r="X13" s="77"/>
-      <c r="Y13" s="77"/>
-      <c r="Z13" s="77"/>
-      <c r="AA13" s="77"/>
-      <c r="AB13" s="78"/>
-      <c r="AC13" s="78"/>
-      <c r="AD13" s="78"/>
-      <c r="AE13" s="78"/>
-      <c r="AF13" s="78"/>
-      <c r="AG13" s="78"/>
-      <c r="AH13" s="78"/>
-      <c r="AI13" s="78"/>
-      <c r="AJ13" s="78"/>
-      <c r="AK13" s="78"/>
-      <c r="AL13" s="78"/>
-      <c r="AM13" s="78"/>
-      <c r="AN13" s="78"/>
-      <c r="AO13" s="78"/>
-      <c r="AP13" s="78"/>
-      <c r="AQ13" s="78"/>
-      <c r="AR13" s="78"/>
-      <c r="AS13" s="71"/>
+      <c r="I13" s="78"/>
+      <c r="J13" s="78"/>
+      <c r="K13" s="78"/>
+      <c r="L13" s="79"/>
+      <c r="M13" s="79"/>
+      <c r="N13" s="79"/>
+      <c r="O13" s="79"/>
+      <c r="P13" s="79"/>
+      <c r="Q13" s="79"/>
+      <c r="R13" s="79"/>
+      <c r="S13" s="79"/>
+      <c r="T13" s="79"/>
+      <c r="U13" s="78"/>
+      <c r="V13" s="78"/>
+      <c r="W13" s="78"/>
+      <c r="X13" s="78"/>
+      <c r="Y13" s="78"/>
+      <c r="Z13" s="78"/>
+      <c r="AA13" s="78"/>
+      <c r="AB13" s="79"/>
+      <c r="AC13" s="79"/>
+      <c r="AD13" s="79"/>
+      <c r="AE13" s="79"/>
+      <c r="AF13" s="79"/>
+      <c r="AG13" s="79"/>
+      <c r="AH13" s="79"/>
+      <c r="AI13" s="79"/>
+      <c r="AJ13" s="79"/>
+      <c r="AK13" s="79"/>
+      <c r="AL13" s="79"/>
+      <c r="AM13" s="79"/>
+      <c r="AN13" s="79"/>
+      <c r="AO13" s="79"/>
+      <c r="AP13" s="79"/>
+      <c r="AQ13" s="79"/>
+      <c r="AR13" s="79"/>
+      <c r="AS13" s="72"/>
     </row>
     <row r="14" spans="1:45">
-      <c r="A14" s="72">
+      <c r="A14" s="73">
         <v>11</v>
       </c>
-      <c r="B14" s="73" t="s">
+      <c r="B14" s="74" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="73" t="s">
+      <c r="C14" s="74" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="74">
+      <c r="D14" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="75">
         <v>37</v>
       </c>
-      <c r="G14" s="75">
+      <c r="G14" s="76">
         <v>89.54</v>
       </c>
-      <c r="H14" s="76">
+      <c r="H14" s="77">
         <f t="shared" si="0"/>
         <v>3312.98</v>
       </c>
-      <c r="I14" s="77"/>
-      <c r="J14" s="77"/>
-      <c r="K14" s="77"/>
-      <c r="L14" s="78"/>
-      <c r="M14" s="78"/>
-      <c r="N14" s="78"/>
-      <c r="O14" s="78"/>
-      <c r="P14" s="78"/>
-      <c r="Q14" s="78"/>
-      <c r="R14" s="78"/>
-      <c r="S14" s="78"/>
-      <c r="T14" s="78"/>
-      <c r="U14" s="77"/>
-      <c r="V14" s="77"/>
-      <c r="W14" s="77"/>
-      <c r="X14" s="77"/>
-      <c r="Y14" s="77"/>
-      <c r="Z14" s="77"/>
-      <c r="AA14" s="77"/>
-      <c r="AB14" s="78"/>
-      <c r="AC14" s="78"/>
-      <c r="AD14" s="78"/>
-      <c r="AE14" s="78"/>
-      <c r="AF14" s="78"/>
-      <c r="AG14" s="78"/>
-      <c r="AH14" s="78"/>
-      <c r="AI14" s="78"/>
-      <c r="AJ14" s="78"/>
-      <c r="AK14" s="78"/>
-      <c r="AL14" s="78"/>
-      <c r="AM14" s="78"/>
-      <c r="AN14" s="78"/>
-      <c r="AO14" s="78"/>
-      <c r="AP14" s="78"/>
-      <c r="AQ14" s="78"/>
-      <c r="AR14" s="78"/>
-      <c r="AS14" s="71"/>
+      <c r="I14" s="78"/>
+      <c r="J14" s="78"/>
+      <c r="K14" s="78"/>
+      <c r="L14" s="79"/>
+      <c r="M14" s="79"/>
+      <c r="N14" s="79"/>
+      <c r="O14" s="79"/>
+      <c r="P14" s="79"/>
+      <c r="Q14" s="79"/>
+      <c r="R14" s="79"/>
+      <c r="S14" s="79"/>
+      <c r="T14" s="79"/>
+      <c r="U14" s="78"/>
+      <c r="V14" s="78"/>
+      <c r="W14" s="78"/>
+      <c r="X14" s="78"/>
+      <c r="Y14" s="78"/>
+      <c r="Z14" s="78"/>
+      <c r="AA14" s="78"/>
+      <c r="AB14" s="79"/>
+      <c r="AC14" s="79"/>
+      <c r="AD14" s="79"/>
+      <c r="AE14" s="79"/>
+      <c r="AF14" s="79"/>
+      <c r="AG14" s="79"/>
+      <c r="AH14" s="79"/>
+      <c r="AI14" s="79"/>
+      <c r="AJ14" s="79"/>
+      <c r="AK14" s="79"/>
+      <c r="AL14" s="79"/>
+      <c r="AM14" s="79"/>
+      <c r="AN14" s="79"/>
+      <c r="AO14" s="79"/>
+      <c r="AP14" s="79"/>
+      <c r="AQ14" s="79"/>
+      <c r="AR14" s="79"/>
+      <c r="AS14" s="72"/>
     </row>
     <row r="15" spans="1:45">
-      <c r="A15" s="72">
-        <v>12</v>
-      </c>
-      <c r="B15" s="73" t="s">
+      <c r="A15" s="73">
+        <v>12</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="73" t="s">
+      <c r="C15" s="74" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="74">
+      <c r="D15" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="75">
         <v>39</v>
       </c>
-      <c r="G15" s="75">
+      <c r="G15" s="76">
         <v>98.25</v>
       </c>
-      <c r="H15" s="76">
+      <c r="H15" s="77">
         <f t="shared" si="0"/>
         <v>3831.75</v>
       </c>
-      <c r="I15" s="77"/>
-      <c r="J15" s="77"/>
-      <c r="K15" s="77"/>
-      <c r="L15" s="78"/>
-      <c r="M15" s="78"/>
-      <c r="N15" s="78"/>
-      <c r="O15" s="78"/>
-      <c r="P15" s="78"/>
-      <c r="Q15" s="78"/>
-      <c r="R15" s="78"/>
-      <c r="S15" s="78"/>
-      <c r="T15" s="78"/>
-      <c r="U15" s="77"/>
-      <c r="V15" s="77"/>
-      <c r="W15" s="77"/>
-      <c r="X15" s="77"/>
-      <c r="Y15" s="77"/>
-      <c r="Z15" s="77"/>
-      <c r="AA15" s="77"/>
-      <c r="AB15" s="78"/>
-      <c r="AC15" s="78"/>
-      <c r="AD15" s="78"/>
-      <c r="AE15" s="78"/>
-      <c r="AF15" s="78"/>
-      <c r="AG15" s="78"/>
-      <c r="AH15" s="78"/>
-      <c r="AI15" s="78"/>
-      <c r="AJ15" s="78"/>
-      <c r="AK15" s="78"/>
-      <c r="AL15" s="78"/>
-      <c r="AM15" s="78"/>
-      <c r="AN15" s="78"/>
-      <c r="AO15" s="78"/>
-      <c r="AP15" s="78"/>
-      <c r="AQ15" s="78"/>
-      <c r="AR15" s="78"/>
-      <c r="AS15" s="71"/>
+      <c r="I15" s="78"/>
+      <c r="J15" s="78"/>
+      <c r="K15" s="78"/>
+      <c r="L15" s="79"/>
+      <c r="M15" s="79"/>
+      <c r="N15" s="79"/>
+      <c r="O15" s="79"/>
+      <c r="P15" s="79"/>
+      <c r="Q15" s="79"/>
+      <c r="R15" s="79"/>
+      <c r="S15" s="79"/>
+      <c r="T15" s="79"/>
+      <c r="U15" s="78"/>
+      <c r="V15" s="78"/>
+      <c r="W15" s="78"/>
+      <c r="X15" s="78"/>
+      <c r="Y15" s="78"/>
+      <c r="Z15" s="78"/>
+      <c r="AA15" s="78"/>
+      <c r="AB15" s="79"/>
+      <c r="AC15" s="79"/>
+      <c r="AD15" s="79"/>
+      <c r="AE15" s="79"/>
+      <c r="AF15" s="79"/>
+      <c r="AG15" s="79"/>
+      <c r="AH15" s="79"/>
+      <c r="AI15" s="79"/>
+      <c r="AJ15" s="79"/>
+      <c r="AK15" s="79"/>
+      <c r="AL15" s="79"/>
+      <c r="AM15" s="79"/>
+      <c r="AN15" s="79"/>
+      <c r="AO15" s="79"/>
+      <c r="AP15" s="79"/>
+      <c r="AQ15" s="79"/>
+      <c r="AR15" s="79"/>
+      <c r="AS15" s="72"/>
     </row>
     <row r="16" spans="1:45">
-      <c r="A16" s="72">
+      <c r="A16" s="73">
         <v>13</v>
       </c>
-      <c r="B16" s="73" t="s">
+      <c r="B16" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="73" t="s">
+      <c r="C16" s="74" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="74">
+      <c r="D16" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="75">
         <v>70</v>
       </c>
-      <c r="G16" s="75">
+      <c r="G16" s="76">
         <v>102.25</v>
       </c>
-      <c r="H16" s="76">
+      <c r="H16" s="77">
         <f t="shared" si="0"/>
         <v>7157.5</v>
       </c>
-      <c r="I16" s="77"/>
-      <c r="J16" s="77"/>
-      <c r="K16" s="77"/>
-      <c r="L16" s="78"/>
-      <c r="M16" s="78"/>
-      <c r="N16" s="78"/>
-      <c r="O16" s="78"/>
-      <c r="P16" s="78"/>
-      <c r="Q16" s="78"/>
-      <c r="R16" s="78"/>
-      <c r="S16" s="78"/>
-      <c r="T16" s="78"/>
-      <c r="U16" s="77"/>
-      <c r="V16" s="77"/>
-      <c r="W16" s="77"/>
-      <c r="X16" s="77"/>
-      <c r="Y16" s="77"/>
-      <c r="Z16" s="77"/>
-      <c r="AA16" s="77"/>
-      <c r="AB16" s="78"/>
-      <c r="AC16" s="78"/>
-      <c r="AD16" s="78"/>
-      <c r="AE16" s="78"/>
-      <c r="AF16" s="78"/>
-      <c r="AG16" s="78"/>
-      <c r="AH16" s="78"/>
-      <c r="AI16" s="78"/>
-      <c r="AJ16" s="78"/>
-      <c r="AK16" s="78"/>
-      <c r="AL16" s="78"/>
-      <c r="AM16" s="78"/>
-      <c r="AN16" s="78"/>
-      <c r="AO16" s="78"/>
-      <c r="AP16" s="78"/>
-      <c r="AQ16" s="78"/>
-      <c r="AR16" s="78"/>
-      <c r="AS16" s="71"/>
+      <c r="I16" s="78"/>
+      <c r="J16" s="78"/>
+      <c r="K16" s="78"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="79"/>
+      <c r="N16" s="79"/>
+      <c r="O16" s="79"/>
+      <c r="P16" s="79"/>
+      <c r="Q16" s="79"/>
+      <c r="R16" s="79"/>
+      <c r="S16" s="79"/>
+      <c r="T16" s="79"/>
+      <c r="U16" s="78"/>
+      <c r="V16" s="78"/>
+      <c r="W16" s="78"/>
+      <c r="X16" s="78"/>
+      <c r="Y16" s="78"/>
+      <c r="Z16" s="78"/>
+      <c r="AA16" s="78"/>
+      <c r="AB16" s="79"/>
+      <c r="AC16" s="79"/>
+      <c r="AD16" s="79"/>
+      <c r="AE16" s="79"/>
+      <c r="AF16" s="79"/>
+      <c r="AG16" s="79"/>
+      <c r="AH16" s="79"/>
+      <c r="AI16" s="79"/>
+      <c r="AJ16" s="79"/>
+      <c r="AK16" s="79"/>
+      <c r="AL16" s="79"/>
+      <c r="AM16" s="79"/>
+      <c r="AN16" s="79"/>
+      <c r="AO16" s="79"/>
+      <c r="AP16" s="79"/>
+      <c r="AQ16" s="79"/>
+      <c r="AR16" s="79"/>
+      <c r="AS16" s="72"/>
     </row>
     <row r="17" spans="1:69">
-      <c r="A17" s="72">
+      <c r="A17" s="73">
         <v>14</v>
       </c>
-      <c r="B17" s="73" t="s">
+      <c r="B17" s="74" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C17" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="73" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="74">
+      <c r="D17" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="75">
         <v>100</v>
       </c>
-      <c r="G17" s="75">
+      <c r="G17" s="76">
         <v>103.5</v>
       </c>
-      <c r="H17" s="76">
+      <c r="H17" s="77">
         <f t="shared" si="0"/>
         <v>10350</v>
       </c>
-      <c r="I17" s="77"/>
-      <c r="J17" s="77"/>
-      <c r="K17" s="77"/>
-      <c r="L17" s="78"/>
-      <c r="M17" s="78"/>
-      <c r="N17" s="78"/>
-      <c r="O17" s="78"/>
-      <c r="P17" s="78"/>
-      <c r="Q17" s="78"/>
-      <c r="R17" s="78"/>
-      <c r="S17" s="79"/>
-      <c r="T17" s="78"/>
-      <c r="U17" s="77"/>
-      <c r="V17" s="77"/>
-      <c r="W17" s="77"/>
-      <c r="X17" s="77"/>
-      <c r="Y17" s="77"/>
-      <c r="Z17" s="77"/>
-      <c r="AA17" s="77"/>
-      <c r="AB17" s="78"/>
-      <c r="AC17" s="78"/>
-      <c r="AD17" s="78"/>
-      <c r="AE17" s="78"/>
-      <c r="AF17" s="78"/>
-      <c r="AG17" s="78"/>
-      <c r="AH17" s="78"/>
-      <c r="AI17" s="78"/>
-      <c r="AJ17" s="78"/>
-      <c r="AK17" s="78"/>
-      <c r="AL17" s="78"/>
-      <c r="AM17" s="78"/>
-      <c r="AN17" s="78"/>
-      <c r="AO17" s="78"/>
-      <c r="AP17" s="78"/>
-      <c r="AQ17" s="78"/>
-      <c r="AR17" s="78"/>
-      <c r="AS17" s="71"/>
+      <c r="I17" s="78"/>
+      <c r="J17" s="78"/>
+      <c r="K17" s="78"/>
+      <c r="L17" s="79"/>
+      <c r="M17" s="79"/>
+      <c r="N17" s="79"/>
+      <c r="O17" s="79"/>
+      <c r="P17" s="79"/>
+      <c r="Q17" s="79"/>
+      <c r="R17" s="79"/>
+      <c r="S17" s="80"/>
+      <c r="T17" s="79"/>
+      <c r="U17" s="78"/>
+      <c r="V17" s="78"/>
+      <c r="W17" s="78"/>
+      <c r="X17" s="78"/>
+      <c r="Y17" s="78"/>
+      <c r="Z17" s="78"/>
+      <c r="AA17" s="78"/>
+      <c r="AB17" s="79"/>
+      <c r="AC17" s="79"/>
+      <c r="AD17" s="79"/>
+      <c r="AE17" s="79"/>
+      <c r="AF17" s="79"/>
+      <c r="AG17" s="79"/>
+      <c r="AH17" s="79"/>
+      <c r="AI17" s="79"/>
+      <c r="AJ17" s="79"/>
+      <c r="AK17" s="79"/>
+      <c r="AL17" s="79"/>
+      <c r="AM17" s="79"/>
+      <c r="AN17" s="79"/>
+      <c r="AO17" s="79"/>
+      <c r="AP17" s="79"/>
+      <c r="AQ17" s="79"/>
+      <c r="AR17" s="79"/>
+      <c r="AS17" s="72"/>
     </row>
     <row r="18" ht="15.25" spans="1:69">
-      <c r="A18" s="80">
+      <c r="A18" s="81">
         <v>15</v>
       </c>
-      <c r="B18" s="81" t="s">
+      <c r="B18" s="82" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="81" t="s">
+      <c r="C18" s="82" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="81" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="81" t="s">
-        <v>12</v>
-      </c>
-      <c r="F18" s="82">
+      <c r="D18" s="82" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="82" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="83">
         <v>85</v>
       </c>
-      <c r="G18" s="83">
+      <c r="G18" s="84">
         <v>65.48</v>
       </c>
-      <c r="H18" s="84">
+      <c r="H18" s="85">
         <f t="shared" si="0"/>
         <v>5565.8</v>
       </c>
-      <c r="I18" s="77"/>
-      <c r="J18" s="77"/>
-      <c r="K18" s="77"/>
-      <c r="L18" s="78"/>
-      <c r="M18" s="78"/>
-      <c r="N18" s="78"/>
-      <c r="O18" s="78"/>
-      <c r="P18" s="78"/>
-      <c r="Q18" s="78"/>
-      <c r="R18" s="78"/>
-      <c r="S18" s="78"/>
-      <c r="T18" s="78"/>
-      <c r="U18" s="77"/>
-      <c r="V18" s="77"/>
-      <c r="W18" s="77"/>
-      <c r="X18" s="77"/>
-      <c r="Y18" s="77"/>
-      <c r="Z18" s="77"/>
-      <c r="AA18" s="77"/>
-      <c r="AB18" s="78"/>
-      <c r="AC18" s="78"/>
-      <c r="AD18" s="78"/>
-      <c r="AE18" s="78"/>
-      <c r="AF18" s="78"/>
-      <c r="AG18" s="78"/>
-      <c r="AH18" s="78"/>
-      <c r="AI18" s="78"/>
-      <c r="AJ18" s="78"/>
-      <c r="AK18" s="78"/>
-      <c r="AL18" s="78"/>
-      <c r="AM18" s="78"/>
-      <c r="AN18" s="78"/>
-      <c r="AO18" s="78"/>
-      <c r="AP18" s="78"/>
-      <c r="AQ18" s="78"/>
-      <c r="AR18" s="78"/>
-      <c r="AS18" s="71"/>
+      <c r="I18" s="78"/>
+      <c r="J18" s="78"/>
+      <c r="K18" s="78"/>
+      <c r="L18" s="79"/>
+      <c r="M18" s="79"/>
+      <c r="N18" s="79"/>
+      <c r="O18" s="79"/>
+      <c r="P18" s="79"/>
+      <c r="Q18" s="79"/>
+      <c r="R18" s="79"/>
+      <c r="S18" s="79"/>
+      <c r="T18" s="79"/>
+      <c r="U18" s="78"/>
+      <c r="V18" s="78"/>
+      <c r="W18" s="78"/>
+      <c r="X18" s="78"/>
+      <c r="Y18" s="78"/>
+      <c r="Z18" s="78"/>
+      <c r="AA18" s="78"/>
+      <c r="AB18" s="79"/>
+      <c r="AC18" s="79"/>
+      <c r="AD18" s="79"/>
+      <c r="AE18" s="79"/>
+      <c r="AF18" s="79"/>
+      <c r="AG18" s="79"/>
+      <c r="AH18" s="79"/>
+      <c r="AI18" s="79"/>
+      <c r="AJ18" s="79"/>
+      <c r="AK18" s="79"/>
+      <c r="AL18" s="79"/>
+      <c r="AM18" s="79"/>
+      <c r="AN18" s="79"/>
+      <c r="AO18" s="79"/>
+      <c r="AP18" s="79"/>
+      <c r="AQ18" s="79"/>
+      <c r="AR18" s="79"/>
+      <c r="AS18" s="72"/>
     </row>
     <row r="19" ht="15.25" spans="1:69">
-      <c r="A19" s="71"/>
+      <c r="A19" s="72"/>
       <c r="B19" s="23" t="s">
         <v>41</v>
       </c>
@@ -3198,92 +3204,92 @@
         <f>SUM(H4:H18)</f>
         <v>71856.76</v>
       </c>
-      <c r="I19" s="85"/>
-      <c r="J19" s="85"/>
-      <c r="K19" s="85"/>
-      <c r="L19" s="85"/>
-      <c r="M19" s="85"/>
-      <c r="N19" s="85"/>
-      <c r="O19" s="85"/>
-      <c r="P19" s="85"/>
-      <c r="Q19" s="85"/>
-      <c r="R19" s="86"/>
-      <c r="S19" s="86"/>
-      <c r="T19" s="86"/>
-      <c r="U19" s="86"/>
-      <c r="V19" s="86"/>
-      <c r="W19" s="86"/>
-      <c r="X19" s="86"/>
-      <c r="Y19" s="86"/>
-      <c r="Z19" s="86"/>
-      <c r="AA19" s="86"/>
-      <c r="AB19" s="86"/>
-      <c r="AC19" s="86"/>
-      <c r="AD19" s="86"/>
-      <c r="AE19" s="86"/>
-      <c r="AF19" s="86"/>
-      <c r="AG19" s="86"/>
-      <c r="AH19" s="86"/>
-      <c r="AI19" s="86"/>
-      <c r="AJ19" s="86"/>
-      <c r="AK19" s="86"/>
-      <c r="AL19" s="86"/>
-      <c r="AM19" s="86"/>
-      <c r="AN19" s="86"/>
-      <c r="AO19" s="86"/>
-      <c r="AP19" s="86"/>
-      <c r="AQ19" s="86"/>
-      <c r="AR19" s="86"/>
-      <c r="AS19" s="71"/>
+      <c r="I19" s="86"/>
+      <c r="J19" s="86"/>
+      <c r="K19" s="86"/>
+      <c r="L19" s="86"/>
+      <c r="M19" s="86"/>
+      <c r="N19" s="86"/>
+      <c r="O19" s="86"/>
+      <c r="P19" s="86"/>
+      <c r="Q19" s="86"/>
+      <c r="R19" s="87"/>
+      <c r="S19" s="87"/>
+      <c r="T19" s="87"/>
+      <c r="U19" s="87"/>
+      <c r="V19" s="87"/>
+      <c r="W19" s="87"/>
+      <c r="X19" s="87"/>
+      <c r="Y19" s="87"/>
+      <c r="Z19" s="87"/>
+      <c r="AA19" s="87"/>
+      <c r="AB19" s="87"/>
+      <c r="AC19" s="87"/>
+      <c r="AD19" s="87"/>
+      <c r="AE19" s="87"/>
+      <c r="AF19" s="87"/>
+      <c r="AG19" s="87"/>
+      <c r="AH19" s="87"/>
+      <c r="AI19" s="87"/>
+      <c r="AJ19" s="87"/>
+      <c r="AK19" s="87"/>
+      <c r="AL19" s="87"/>
+      <c r="AM19" s="87"/>
+      <c r="AN19" s="87"/>
+      <c r="AO19" s="87"/>
+      <c r="AP19" s="87"/>
+      <c r="AQ19" s="87"/>
+      <c r="AR19" s="87"/>
+      <c r="AS19" s="72"/>
     </row>
     <row r="20" s="1" customFormat="1" spans="1:69">
-      <c r="A20" s="87" t="s">
+      <c r="A20" s="88" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="87"/>
-      <c r="C20" s="87"/>
-      <c r="D20" s="87"/>
-      <c r="E20" s="87"/>
-      <c r="F20" s="87"/>
-      <c r="G20" s="87"/>
-      <c r="H20" s="87"/>
-      <c r="I20" s="88"/>
-      <c r="J20" s="88"/>
-      <c r="K20" s="88"/>
-      <c r="L20" s="88"/>
-      <c r="M20" s="88"/>
-      <c r="N20" s="88"/>
-      <c r="O20" s="88"/>
-      <c r="P20" s="88"/>
-      <c r="Q20" s="88"/>
-      <c r="R20" s="87"/>
-      <c r="S20" s="87"/>
-      <c r="T20" s="87"/>
-      <c r="U20" s="87"/>
-      <c r="V20" s="87"/>
-      <c r="W20" s="87"/>
-      <c r="X20" s="87"/>
-      <c r="Y20" s="87"/>
-      <c r="Z20" s="87"/>
-      <c r="AA20" s="87"/>
-      <c r="AB20" s="87"/>
-      <c r="AC20" s="87"/>
-      <c r="AD20" s="87"/>
-      <c r="AE20" s="87"/>
-      <c r="AF20" s="87"/>
-      <c r="AG20" s="87"/>
-      <c r="AH20" s="87"/>
-      <c r="AI20" s="87"/>
-      <c r="AJ20" s="87"/>
-      <c r="AK20" s="87"/>
-      <c r="AL20" s="87"/>
-      <c r="AM20" s="87"/>
-      <c r="AN20" s="87"/>
-      <c r="AO20" s="87"/>
-      <c r="AP20" s="87"/>
-      <c r="AQ20" s="87"/>
-      <c r="AR20" s="87"/>
-      <c r="AS20" s="89"/>
+      <c r="B20" s="88"/>
+      <c r="C20" s="88"/>
+      <c r="D20" s="88"/>
+      <c r="E20" s="88"/>
+      <c r="F20" s="88"/>
+      <c r="G20" s="88"/>
+      <c r="H20" s="88"/>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="89"/>
+      <c r="L20" s="89"/>
+      <c r="M20" s="89"/>
+      <c r="N20" s="89"/>
+      <c r="O20" s="89"/>
+      <c r="P20" s="89"/>
+      <c r="Q20" s="89"/>
+      <c r="R20" s="88"/>
+      <c r="S20" s="88"/>
+      <c r="T20" s="88"/>
+      <c r="U20" s="88"/>
+      <c r="V20" s="88"/>
+      <c r="W20" s="88"/>
+      <c r="X20" s="88"/>
+      <c r="Y20" s="88"/>
+      <c r="Z20" s="88"/>
+      <c r="AA20" s="88"/>
+      <c r="AB20" s="88"/>
+      <c r="AC20" s="88"/>
+      <c r="AD20" s="88"/>
+      <c r="AE20" s="88"/>
+      <c r="AF20" s="88"/>
+      <c r="AG20" s="88"/>
+      <c r="AH20" s="88"/>
+      <c r="AI20" s="88"/>
+      <c r="AJ20" s="88"/>
+      <c r="AK20" s="88"/>
+      <c r="AL20" s="88"/>
+      <c r="AM20" s="88"/>
+      <c r="AN20" s="88"/>
+      <c r="AO20" s="88"/>
+      <c r="AP20" s="88"/>
+      <c r="AQ20" s="88"/>
+      <c r="AR20" s="88"/>
+      <c r="AS20" s="90"/>
     </row>
     <row r="21" s="1" customFormat="1" spans="1:69">
       <c r="A21" s="28" t="s">
@@ -3354,33 +3360,33 @@
       <c r="AP21" s="30"/>
       <c r="AQ21" s="30"/>
       <c r="AR21" s="30"/>
-      <c r="AS21" s="90"/>
-      <c r="AT21" s="91"/>
-      <c r="AU21" s="91"/>
-      <c r="AV21" s="91"/>
-      <c r="AW21" s="91"/>
-      <c r="AX21" s="91"/>
-      <c r="AY21" s="91"/>
-      <c r="AZ21" s="91"/>
-      <c r="BA21" s="91"/>
-      <c r="BB21" s="91"/>
-      <c r="BC21" s="91"/>
-      <c r="BD21" s="91"/>
-      <c r="BE21" s="91"/>
-      <c r="BF21" s="91"/>
-      <c r="BG21" s="91"/>
-      <c r="BH21" s="91"/>
-      <c r="BI21" s="91"/>
-      <c r="BJ21" s="91"/>
-      <c r="BK21" s="91"/>
-      <c r="BL21" s="91"/>
-      <c r="BM21" s="91"/>
-      <c r="BN21" s="91"/>
-      <c r="BO21" s="91"/>
-      <c r="BP21" s="91"/>
-      <c r="BQ21" s="91"/>
+      <c r="AS21" s="91"/>
+      <c r="AT21" s="92"/>
+      <c r="AU21" s="92"/>
+      <c r="AV21" s="92"/>
+      <c r="AW21" s="92"/>
+      <c r="AX21" s="92"/>
+      <c r="AY21" s="92"/>
+      <c r="AZ21" s="92"/>
+      <c r="BA21" s="92"/>
+      <c r="BB21" s="92"/>
+      <c r="BC21" s="92"/>
+      <c r="BD21" s="92"/>
+      <c r="BE21" s="92"/>
+      <c r="BF21" s="92"/>
+      <c r="BG21" s="92"/>
+      <c r="BH21" s="92"/>
+      <c r="BI21" s="92"/>
+      <c r="BJ21" s="92"/>
+      <c r="BK21" s="92"/>
+      <c r="BL21" s="92"/>
+      <c r="BM21" s="92"/>
+      <c r="BN21" s="92"/>
+      <c r="BO21" s="92"/>
+      <c r="BP21" s="92"/>
+      <c r="BQ21" s="92"/>
     </row>
-    <row r="22" s="55" customFormat="1" ht="15.25" spans="1:69">
+    <row r="22" s="56" customFormat="1" ht="15.25" spans="1:69">
       <c r="A22" s="34" t="s">
         <v>2</v>
       </c>
@@ -3414,22 +3420,22 @@
       <c r="K22" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="L22" s="92" t="s">
+      <c r="L22" s="93" t="s">
         <v>55</v>
       </c>
-      <c r="M22" s="92" t="s">
+      <c r="M22" s="93" t="s">
         <v>56</v>
       </c>
-      <c r="N22" s="92" t="s">
+      <c r="N22" s="93" t="s">
         <v>57</v>
       </c>
-      <c r="O22" s="92" t="s">
+      <c r="O22" s="93" t="s">
         <v>58</v>
       </c>
-      <c r="P22" s="92" t="s">
+      <c r="P22" s="93" t="s">
         <v>59</v>
       </c>
-      <c r="Q22" s="92" t="s">
+      <c r="Q22" s="93" t="s">
         <v>60</v>
       </c>
       <c r="R22" s="35" t="s">
@@ -3519,63 +3525,63 @@
       <c r="AT22" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="AU22" s="91"/>
-      <c r="AV22" s="91"/>
-      <c r="AW22" s="93" t="s">
+      <c r="AU22" s="92"/>
+      <c r="AV22" s="92"/>
+      <c r="AW22" s="94" t="s">
         <v>89</v>
       </c>
-      <c r="AX22" s="93" t="s">
+      <c r="AX22" s="94" t="s">
         <v>90</v>
       </c>
-      <c r="AY22" s="93" t="s">
+      <c r="AY22" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AZ22" s="91"/>
-      <c r="BA22" s="93" t="s">
+      <c r="AZ22" s="92"/>
+      <c r="BA22" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="BB22" s="93" t="s">
+      <c r="BB22" s="94" t="s">
         <v>93</v>
       </c>
-      <c r="BC22" s="93" t="s">
+      <c r="BC22" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="BD22" s="93" t="s">
+      <c r="BD22" s="94" t="s">
         <v>95</v>
       </c>
-      <c r="BE22" s="93" t="s">
+      <c r="BE22" s="94" t="s">
         <v>96</v>
       </c>
-      <c r="BF22" s="93" t="s">
+      <c r="BF22" s="94" t="s">
         <v>97</v>
       </c>
-      <c r="BG22" s="93" t="s">
+      <c r="BG22" s="94" t="s">
         <v>98</v>
       </c>
-      <c r="BH22" s="93" t="s">
+      <c r="BH22" s="94" t="s">
         <v>99</v>
       </c>
-      <c r="BI22" s="93" t="s">
+      <c r="BI22" s="94" t="s">
         <v>100</v>
       </c>
-      <c r="BJ22" s="93" t="s">
+      <c r="BJ22" s="94" t="s">
         <v>101</v>
       </c>
-      <c r="BK22" s="93" t="s">
+      <c r="BK22" s="94" t="s">
         <v>102</v>
       </c>
-      <c r="BL22" s="93" t="s">
+      <c r="BL22" s="94" t="s">
         <v>103</v>
       </c>
-      <c r="BM22" s="91"/>
-      <c r="BN22" s="91"/>
-      <c r="BO22" s="93" t="s">
+      <c r="BM22" s="92"/>
+      <c r="BN22" s="92"/>
+      <c r="BO22" s="94" t="s">
         <v>104</v>
       </c>
-      <c r="BP22" s="93" t="s">
+      <c r="BP22" s="94" t="s">
         <v>105</v>
       </c>
-      <c r="BQ22" s="93" t="s">
+      <c r="BQ22" s="94" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3601,52 +3607,52 @@
       <c r="G23" s="41">
         <v>100</v>
       </c>
-      <c r="H23" s="94">
+      <c r="H23" s="95">
         <f>F23*G23</f>
         <v>200</v>
       </c>
-      <c r="I23" s="91">
+      <c r="I23" s="92">
         <v>1</v>
       </c>
-      <c r="J23" s="94">
+      <c r="J23" s="95">
         <v>2</v>
       </c>
-      <c r="K23" s="94">
+      <c r="K23" s="95">
         <v>4</v>
       </c>
-      <c r="L23" s="94">
+      <c r="L23" s="95">
         <f>H23</f>
         <v>200</v>
       </c>
-      <c r="M23" s="94">
+      <c r="M23" s="95">
         <f>ROUND(L23*I23%,2)</f>
         <v>2</v>
       </c>
-      <c r="N23" s="94">
+      <c r="N23" s="95">
         <f>H23-M23</f>
         <v>198</v>
       </c>
-      <c r="O23" s="94">
+      <c r="O23" s="95">
         <f>ROUND(N23*J23%,2)</f>
         <v>3.96</v>
       </c>
-      <c r="P23" s="94">
+      <c r="P23" s="95">
         <f>ROUND(N23-O23,2)</f>
         <v>194.04</v>
       </c>
-      <c r="Q23" s="94">
+      <c r="Q23" s="95">
         <f>ROUND(P23*K23%,2)</f>
         <v>7.76</v>
       </c>
-      <c r="R23" s="94">
+      <c r="R23" s="95">
         <f>M23+O23+Q23</f>
         <v>13.72</v>
       </c>
-      <c r="S23" s="94">
+      <c r="S23" s="95">
         <f>(H23-R23)</f>
         <v>186.28</v>
       </c>
-      <c r="T23" s="94" t="s">
+      <c r="T23" s="95" t="s">
         <v>107</v>
       </c>
       <c r="U23" s="44">
@@ -3679,68 +3685,68 @@
         <f>V23+W23+X23+Y23+AA23</f>
         <v>0</v>
       </c>
-      <c r="AC23" s="94">
+      <c r="AC23" s="95">
         <f>IF($V21=1,S23+AB23,S23)</f>
         <v>186.28</v>
       </c>
-      <c r="AD23" s="94">
+      <c r="AD23" s="95">
         <v>120</v>
       </c>
-      <c r="AE23" s="94">
+      <c r="AE23" s="95">
         <f>IF($P$21=1,(S23/$S$24)*$E$35,AD23/$AD$24*$E$35)</f>
         <v>0</v>
       </c>
-      <c r="AF23" s="94"/>
-      <c r="AG23" s="94">
+      <c r="AF23" s="95"/>
+      <c r="AG23" s="95">
         <f>IF($P$21=1,(S23/$S$24)*$E$37,AD23/$AD$24*$E$37)</f>
         <v>0</v>
       </c>
-      <c r="AH23" s="94">
+      <c r="AH23" s="95">
         <f>IF($P$21=1,(S23/$S$24)*$E$37,AD23/$AD$24*$E$37)</f>
         <v>0</v>
       </c>
-      <c r="AI23" s="94">
+      <c r="AI23" s="95">
         <f>S23*$M$21</f>
         <v>15833.8</v>
       </c>
-      <c r="AJ23" s="94">
+      <c r="AJ23" s="95">
         <f>IF($C$21=3,0,AG23+AH23)</f>
         <v>0</v>
       </c>
-      <c r="AK23" s="94">
+      <c r="AK23" s="95">
         <f>IF($C$21=3,AE23+AG23+AH23,0)</f>
         <v>0</v>
       </c>
-      <c r="AL23" s="94">
+      <c r="AL23" s="95">
         <v>1</v>
       </c>
-      <c r="AM23" s="94">
+      <c r="AM23" s="95">
         <f>F23/AL23</f>
         <v>2</v>
       </c>
-      <c r="AN23" s="94">
+      <c r="AN23" s="95">
         <f>AI23/AM23</f>
         <v>7916.9</v>
       </c>
-      <c r="AO23" s="94">
+      <c r="AO23" s="95">
         <f>AJ23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AP23" s="94">
+      <c r="AP23" s="95">
         <f>AK23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AQ23" s="94" t="s">
-        <v>12</v>
-      </c>
-      <c r="AR23" s="94">
+      <c r="AQ23" s="95" t="s">
+        <v>12</v>
+      </c>
+      <c r="AR23" s="95">
         <f>AN23+AO23+AP23</f>
         <v>7916.9</v>
       </c>
-      <c r="AS23" s="94" t="s">
+      <c r="AS23" s="95" t="s">
         <v>108</v>
       </c>
-      <c r="AT23" s="94" t="s">
+      <c r="AT23" s="95" t="s">
         <v>12</v>
       </c>
       <c r="AU23" t="s">
@@ -3749,41 +3755,41 @@
       <c r="AV23" t="s">
         <v>110</v>
       </c>
-      <c r="AW23" s="94">
+      <c r="AW23" s="95">
         <f>AM23</f>
         <v>2</v>
       </c>
-      <c r="AX23" s="94">
+      <c r="AX23" s="95">
         <f>AR23</f>
         <v>7916.9</v>
       </c>
-      <c r="AY23" s="94">
+      <c r="AY23" s="95">
         <f>AU23+AW23</f>
         <v>2</v>
       </c>
       <c r="AZ23" t="s">
         <v>110</v>
       </c>
-      <c r="BA23" s="95"/>
-      <c r="BB23" s="95" t="s">
+      <c r="BA23" s="96"/>
+      <c r="BB23" s="96" t="s">
         <v>111</v>
       </c>
-      <c r="BC23" s="95" t="s">
+      <c r="BC23" s="96" t="s">
         <v>112</v>
       </c>
-      <c r="BD23" s="96" t="s">
+      <c r="BD23" s="97" t="s">
         <v>113</v>
       </c>
-      <c r="BE23" s="96" t="s">
+      <c r="BE23" s="97" t="s">
         <v>114</v>
       </c>
-      <c r="BF23" s="95"/>
-      <c r="BG23" s="95"/>
-      <c r="BH23" s="95"/>
-      <c r="BI23" s="94"/>
-      <c r="BJ23" s="94"/>
-      <c r="BK23" s="94"/>
-      <c r="BL23" s="94" t="s">
+      <c r="BF23" s="96"/>
+      <c r="BG23" s="96"/>
+      <c r="BH23" s="96"/>
+      <c r="BI23" s="95"/>
+      <c r="BJ23" s="95"/>
+      <c r="BK23" s="95"/>
+      <c r="BL23" s="95" t="s">
         <v>115</v>
       </c>
       <c r="BM23" t="s">
@@ -3792,73 +3798,73 @@
       <c r="BN23" t="s">
         <v>117</v>
       </c>
-      <c r="BO23" s="94">
+      <c r="BO23" s="95">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>3958.4505</v>
       </c>
-      <c r="BP23" s="95">
+      <c r="BP23" s="96">
         <f>BN23+AW23</f>
         <v>2</v>
       </c>
-      <c r="BQ23" s="95">
+      <c r="BQ23" s="96">
         <v>88363222</v>
       </c>
     </row>
     <row r="24" s="1" customFormat="1" spans="1:69">
-      <c r="A24" s="90"/>
-      <c r="B24" s="91"/>
-      <c r="C24" s="91"/>
-      <c r="D24" s="97" t="s">
+      <c r="A24" s="91"/>
+      <c r="B24" s="92"/>
+      <c r="C24" s="92"/>
+      <c r="D24" s="98" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="97"/>
-      <c r="F24" s="97"/>
-      <c r="G24" s="97"/>
-      <c r="H24" s="97">
+      <c r="E24" s="98"/>
+      <c r="F24" s="98"/>
+      <c r="G24" s="98"/>
+      <c r="H24" s="98">
         <f>SUM(H23:H23)</f>
         <v>200</v>
       </c>
-      <c r="I24" s="90"/>
-      <c r="J24" s="90"/>
-      <c r="K24" s="90"/>
-      <c r="L24" s="90"/>
-      <c r="M24" s="90"/>
-      <c r="N24" s="90"/>
-      <c r="O24" s="90"/>
-      <c r="P24" s="90"/>
-      <c r="Q24" s="90"/>
-      <c r="R24" s="97">
+      <c r="I24" s="91"/>
+      <c r="J24" s="91"/>
+      <c r="K24" s="91"/>
+      <c r="L24" s="91"/>
+      <c r="M24" s="91"/>
+      <c r="N24" s="91"/>
+      <c r="O24" s="91"/>
+      <c r="P24" s="91"/>
+      <c r="Q24" s="91"/>
+      <c r="R24" s="98">
         <f t="shared" ref="R24:Y24" si="1">SUM(R23:R23)</f>
         <v>13.72</v>
       </c>
-      <c r="S24" s="98">
+      <c r="S24" s="99">
         <f t="shared" si="1"/>
         <v>186.28</v>
       </c>
-      <c r="T24" s="97"/>
-      <c r="U24" s="97"/>
-      <c r="V24" s="99">
+      <c r="T24" s="98"/>
+      <c r="U24" s="98"/>
+      <c r="V24" s="100">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="W24" s="99">
+      <c r="W24" s="100">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="X24" s="99">
+      <c r="X24" s="100">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Y24" s="99">
+      <c r="Y24" s="100">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Z24" s="99"/>
-      <c r="AA24" s="99">
+      <c r="Z24" s="100"/>
+      <c r="AA24" s="100">
         <f t="shared" ref="AA24:AE24" si="2">SUM(AA23:AA23)</f>
         <v>0</v>
       </c>
-      <c r="AB24" s="97">
+      <c r="AB24" s="98">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -3866,32 +3872,32 @@
         <f t="shared" si="2"/>
         <v>186.28</v>
       </c>
-      <c r="AD24" s="100">
+      <c r="AD24" s="101">
         <f t="shared" si="2"/>
         <v>120</v>
       </c>
-      <c r="AE24" s="100">
+      <c r="AE24" s="101">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF24" s="38"/>
-      <c r="AG24" s="100">
+      <c r="AG24" s="101">
         <f>SUM(AG23:AG23)</f>
         <v>0</v>
       </c>
-      <c r="AH24" s="100">
+      <c r="AH24" s="101">
         <f t="shared" ref="AG24:AK24" si="3">SUM(AH23:AH23)</f>
         <v>0</v>
       </c>
-      <c r="AI24" s="100">
+      <c r="AI24" s="101">
         <f t="shared" si="3"/>
         <v>15833.8</v>
       </c>
-      <c r="AJ24" s="100">
+      <c r="AJ24" s="101">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AK24" s="100">
+      <c r="AK24" s="101">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3902,31 +3908,31 @@
       <c r="AP24" s="38"/>
       <c r="AQ24" s="38"/>
       <c r="AR24" s="38"/>
-      <c r="AS24" s="90"/>
-      <c r="AT24" s="91"/>
-      <c r="AU24" s="91"/>
-      <c r="AV24" s="91"/>
-      <c r="AW24" s="91"/>
-      <c r="AX24" s="91"/>
-      <c r="AY24" s="91"/>
-      <c r="AZ24" s="91"/>
-      <c r="BA24" s="91"/>
-      <c r="BB24" s="91"/>
-      <c r="BC24" s="91"/>
-      <c r="BD24" s="91"/>
-      <c r="BE24" s="91"/>
-      <c r="BF24" s="91"/>
-      <c r="BG24" s="91"/>
-      <c r="BH24" s="91"/>
-      <c r="BI24" s="91"/>
-      <c r="BJ24" s="91"/>
-      <c r="BK24" s="91"/>
-      <c r="BL24" s="91"/>
-      <c r="BM24" s="91"/>
-      <c r="BN24" s="91"/>
-      <c r="BO24" s="91"/>
-      <c r="BP24" s="91"/>
-      <c r="BQ24" s="91"/>
+      <c r="AS24" s="91"/>
+      <c r="AT24" s="92"/>
+      <c r="AU24" s="92"/>
+      <c r="AV24" s="92"/>
+      <c r="AW24" s="92"/>
+      <c r="AX24" s="92"/>
+      <c r="AY24" s="92"/>
+      <c r="AZ24" s="92"/>
+      <c r="BA24" s="92"/>
+      <c r="BB24" s="92"/>
+      <c r="BC24" s="92"/>
+      <c r="BD24" s="92"/>
+      <c r="BE24" s="92"/>
+      <c r="BF24" s="92"/>
+      <c r="BG24" s="92"/>
+      <c r="BH24" s="92"/>
+      <c r="BI24" s="92"/>
+      <c r="BJ24" s="92"/>
+      <c r="BK24" s="92"/>
+      <c r="BL24" s="92"/>
+      <c r="BM24" s="92"/>
+      <c r="BN24" s="92"/>
+      <c r="BO24" s="92"/>
+      <c r="BP24" s="92"/>
+      <c r="BQ24" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5745,7 +5751,7 @@
       <c r="BP21" s="33"/>
       <c r="BQ21" s="33"/>
     </row>
-    <row r="22" s="55" customFormat="1" ht="15.25" spans="1:69">
+    <row r="22" s="56" customFormat="1" ht="15.25" spans="1:69">
       <c r="A22" s="34" t="s">
         <v>2</v>
       </c>
@@ -5779,22 +5785,22 @@
       <c r="K22" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L22" s="60" t="s">
+      <c r="L22" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="M22" s="60" t="s">
+      <c r="M22" s="61" t="s">
         <v>56</v>
       </c>
-      <c r="N22" s="60" t="s">
+      <c r="N22" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="O22" s="60" t="s">
+      <c r="O22" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="P22" s="60" t="s">
+      <c r="P22" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="Q22" s="60" t="s">
+      <c r="Q22" s="61" t="s">
         <v>58</v>
       </c>
       <c r="R22" s="35" t="s">
@@ -5958,10 +5964,10 @@
       <c r="A23" s="28">
         <v>1</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="55" t="s">
         <v>126</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="55" t="s">
         <v>126</v>
       </c>
       <c r="D23" s="28" t="s">
@@ -6013,7 +6019,7 @@
         <f>ROUND(P23*K23%,2)</f>
         <v>7.76</v>
       </c>
-      <c r="R23" s="61">
+      <c r="R23" s="62">
         <f>ROUND(M23+O23+Q23,3)</f>
         <v>13.72</v>
       </c>
@@ -6054,65 +6060,65 @@
         <f>V23+W23+X23+Y23+AA23</f>
         <v>0</v>
       </c>
-      <c r="AC23" s="62">
+      <c r="AC23" s="63">
         <f>IF($V21=1,S23+AB23,S23)</f>
         <v>186.28</v>
       </c>
-      <c r="AD23" s="61">
+      <c r="AD23" s="62">
         <v>120</v>
       </c>
-      <c r="AE23" s="61">
+      <c r="AE23" s="62">
         <f>IF($P$21=1,(S23/$S$23)*$E$30,AD23/$AD$4*$E$30)</f>
         <v>0</v>
       </c>
-      <c r="AF23" s="61"/>
-      <c r="AG23" s="61">
+      <c r="AF23" s="62"/>
+      <c r="AG23" s="62">
         <f>IF($P$21=1,(S23/$S$23)*$E$20,AD23/$AD$23*$E$20)</f>
         <v>0</v>
       </c>
-      <c r="AH23" s="61">
+      <c r="AH23" s="62">
         <f>IF($P$21=1,(S23/$S$23)*$E$21,AD23/$AD$23*$E$21)</f>
         <v>0</v>
       </c>
-      <c r="AI23" s="61">
+      <c r="AI23" s="62">
         <f>S23*$M21</f>
         <v>15833.8</v>
       </c>
-      <c r="AJ23" s="61">
+      <c r="AJ23" s="62">
         <f>IF($C$2=3,0,AG23+AH23)</f>
         <v>0</v>
       </c>
-      <c r="AK23" s="61">
+      <c r="AK23" s="62">
         <f>IF($C$2=3,AE23+AG23+AH23,0)</f>
         <v>0</v>
       </c>
-      <c r="AL23" s="63">
+      <c r="AL23" s="64">
         <v>3</v>
       </c>
-      <c r="AM23" s="61">
+      <c r="AM23" s="62">
         <f>F23/AL23</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="AN23" s="61">
+      <c r="AN23" s="62">
         <f>ROUND(AI23/AM23,5)</f>
         <v>23750.7</v>
       </c>
-      <c r="AO23" s="61">
+      <c r="AO23" s="62">
         <f>AJ23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AP23" s="61">
+      <c r="AP23" s="62">
         <f>AK23/AM23</f>
         <v>0</v>
       </c>
-      <c r="AQ23" s="61" t="s">
-        <v>12</v>
-      </c>
-      <c r="AR23" s="61">
+      <c r="AQ23" s="62" t="s">
+        <v>12</v>
+      </c>
+      <c r="AR23" s="62">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>23750.7</v>
       </c>
-      <c r="AS23" s="64" t="s">
+      <c r="AS23" s="65" t="s">
         <v>127</v>
       </c>
       <c r="AT23" s="54" t="s">
@@ -6128,7 +6134,7 @@
         <f>AM23</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="AX23" s="61">
+      <c r="AX23" s="62">
         <f>AR23</f>
         <v>23750.7</v>
       </c>
@@ -6136,30 +6142,30 @@
         <f>AU23+AW23</f>
         <v>117.000666666667</v>
       </c>
-      <c r="AZ23" s="65">
+      <c r="AZ23" s="66">
         <f>ROUND(((AU23*AV23)+(AW23*AX23))/(AU23+AW23),5)</f>
         <v>6394.32854</v>
       </c>
-      <c r="BA23" s="66"/>
-      <c r="BB23" s="66" t="s">
+      <c r="BA23" s="67"/>
+      <c r="BB23" s="67" t="s">
         <v>111</v>
       </c>
-      <c r="BC23" s="66" t="s">
+      <c r="BC23" s="67" t="s">
         <v>112</v>
       </c>
-      <c r="BD23" s="67" t="s">
+      <c r="BD23" s="68" t="s">
         <v>113</v>
       </c>
-      <c r="BE23" s="67" t="s">
+      <c r="BE23" s="68" t="s">
         <v>114</v>
       </c>
-      <c r="BF23" s="66"/>
-      <c r="BG23" s="66"/>
-      <c r="BH23" s="66"/>
+      <c r="BF23" s="67"/>
+      <c r="BG23" s="67"/>
+      <c r="BH23" s="67"/>
       <c r="BI23" s="54"/>
       <c r="BJ23" s="54"/>
       <c r="BK23" s="54"/>
-      <c r="BL23" s="68" t="s">
+      <c r="BL23" s="69" t="s">
         <v>115</v>
       </c>
       <c r="BM23" s="43" t="s">
@@ -6172,11 +6178,11 @@
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>280.32668</v>
       </c>
-      <c r="BP23" s="66">
+      <c r="BP23" s="67">
         <f>ROUND(BN23+AW23,3)</f>
         <v>120.667</v>
       </c>
-      <c r="BQ23" s="69">
+      <c r="BQ23" s="70">
         <v>123562</v>
       </c>
     </row>
@@ -8332,10 +8338,10 @@
       <c r="A23" s="28">
         <v>1</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="55" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="55" t="s">
         <v>134</v>
       </c>
       <c r="D23" s="28" t="s">
@@ -8348,11 +8354,11 @@
         <v>2</v>
       </c>
       <c r="G23" s="41">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="H23" s="42">
         <f>F23*G23</f>
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I23" s="43">
         <v>1</v>
@@ -8365,35 +8371,35 @@
       </c>
       <c r="L23" s="42">
         <f>H23</f>
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="M23" s="42">
         <f>ROUND(L23*I23%,2)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N23" s="42">
         <f>H23-M23</f>
-        <v>198</v>
+        <v>495</v>
       </c>
       <c r="O23" s="42">
         <f>ROUND(N23*J23%,2)</f>
-        <v>3.96</v>
+        <v>9.9</v>
       </c>
       <c r="P23" s="42">
         <f>ROUND(N23-O23,2)</f>
-        <v>194.04</v>
+        <v>485.1</v>
       </c>
       <c r="Q23" s="42">
         <f>ROUND(P23*K23%,2)</f>
-        <v>7.76</v>
+        <v>19.4</v>
       </c>
       <c r="R23" s="42">
         <f>M23+O23+Q23</f>
-        <v>13.72</v>
+        <v>34.3</v>
       </c>
       <c r="S23" s="42">
         <f>(H23-R23)</f>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="T23" s="42" t="s">
         <v>107</v>
@@ -8430,7 +8436,7 @@
       </c>
       <c r="AC23" s="42">
         <f>IF($V21=1,S23+AB23,S23)</f>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="AD23" s="42">
         <v>120</v>
@@ -8450,7 +8456,7 @@
       </c>
       <c r="AI23" s="42">
         <f>S23*$M$21</f>
-        <v>15833.8</v>
+        <v>39584.5</v>
       </c>
       <c r="AJ23" s="42">
         <f>IF($C$21=3,0,AG23+AH23)</f>
@@ -8469,7 +8475,7 @@
       </c>
       <c r="AN23" s="42">
         <f>AI23/AM23</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="AO23" s="42">
         <f>AJ23/AM23</f>
@@ -8484,7 +8490,7 @@
       </c>
       <c r="AR23" s="42">
         <f>AN23+AO23+AP23</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="AS23" s="42" t="s">
         <v>108</v>
@@ -8504,7 +8510,7 @@
       </c>
       <c r="AX23" s="42">
         <f>AR23</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="AY23" s="42">
         <f>AU23+AW23</f>
@@ -8565,7 +8571,7 @@
       <c r="G24" s="49"/>
       <c r="H24" s="49">
         <f>SUM(H23:H23)</f>
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -8578,11 +8584,11 @@
       <c r="Q24" s="32"/>
       <c r="R24" s="49">
         <f t="shared" ref="R24:Y24" si="1">SUM(R23:R23)</f>
-        <v>13.72</v>
+        <v>34.3</v>
       </c>
       <c r="S24" s="50">
         <f t="shared" si="1"/>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="T24" s="49"/>
       <c r="U24" s="49"/>
@@ -8613,7 +8619,7 @@
       </c>
       <c r="AC24" s="52">
         <f t="shared" si="2"/>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="AD24" s="53">
         <f t="shared" si="2"/>
@@ -8634,7 +8640,7 @@
       </c>
       <c r="AI24" s="53">
         <f t="shared" si="3"/>
-        <v>15833.8</v>
+        <v>39584.5</v>
       </c>
       <c r="AJ24" s="53">
         <f t="shared" si="3"/>
@@ -10254,14 +10260,14 @@
     </row>
     <row r="19" ht="15.25" spans="1:69">
       <c r="A19" s="3"/>
-      <c r="B19" s="57" t="s">
+      <c r="B19" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="59"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="60"/>
       <c r="H19" s="24">
         <f>SUM(H4:H18)</f>
         <v>71856.76</v>
@@ -10701,10 +10707,10 @@
       <c r="A23" s="28">
         <v>1</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="55" t="s">
         <v>137</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="55" t="s">
         <v>137</v>
       </c>
       <c r="D23" s="28" t="s">
@@ -10717,11 +10723,11 @@
         <v>2</v>
       </c>
       <c r="G23" s="41">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="H23" s="42">
         <f>F23*G23</f>
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I23" s="43">
         <v>1</v>
@@ -10734,35 +10740,35 @@
       </c>
       <c r="L23" s="42">
         <f>H23</f>
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="M23" s="42">
         <f>ROUND(L23*I23%,2)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N23" s="42">
         <f>H23-M23</f>
-        <v>198</v>
+        <v>495</v>
       </c>
       <c r="O23" s="42">
         <f>ROUND(N23*J23%,2)</f>
-        <v>3.96</v>
+        <v>9.9</v>
       </c>
       <c r="P23" s="42">
         <f>ROUND(N23-O23,2)</f>
-        <v>194.04</v>
+        <v>485.1</v>
       </c>
       <c r="Q23" s="42">
         <f>ROUND(P23*K23%,2)</f>
-        <v>7.76</v>
+        <v>19.4</v>
       </c>
       <c r="R23" s="42">
         <f>M23+O23+Q23</f>
-        <v>13.72</v>
+        <v>34.3</v>
       </c>
       <c r="S23" s="42">
         <f>(H23-R23)</f>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="T23" s="42" t="s">
         <v>107</v>
@@ -10799,7 +10805,7 @@
       </c>
       <c r="AC23" s="42">
         <f>IF($V21=1,S23+AB23,S23)</f>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="AD23" s="42">
         <v>120</v>
@@ -10819,7 +10825,7 @@
       </c>
       <c r="AI23" s="42">
         <f>S23*$M$21</f>
-        <v>15833.8</v>
+        <v>39584.5</v>
       </c>
       <c r="AJ23" s="42">
         <f>IF($C$21=3,0,AG23+AH23)</f>
@@ -10838,7 +10844,7 @@
       </c>
       <c r="AN23" s="42">
         <f>AI23/AM23</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="AO23" s="42">
         <f>AJ23/AM23</f>
@@ -10853,7 +10859,7 @@
       </c>
       <c r="AR23" s="42">
         <f>AN23+AO23+AP23</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="AS23" s="42" t="s">
         <v>108</v>
@@ -10869,7 +10875,7 @@
       </c>
       <c r="AX23" s="42">
         <f>AR23</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="AY23" s="42">
         <f>AU23+AW23</f>
@@ -10877,7 +10883,7 @@
       </c>
       <c r="AZ23" s="42">
         <f>ROUND(((AU23*AV23)+(AW23*AX23))/(AU23+AW23),5)</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="BA23" s="45"/>
       <c r="BB23" s="45" t="s">
@@ -10905,7 +10911,7 @@
       <c r="BN23" s="43"/>
       <c r="BO23" s="42">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>7916.9</v>
+        <v>19792.25</v>
       </c>
       <c r="BP23" s="45">
         <f>BN23+AW23</f>
@@ -10927,7 +10933,7 @@
       <c r="G24" s="49"/>
       <c r="H24" s="49">
         <f>SUM(H23:H23)</f>
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -10940,11 +10946,11 @@
       <c r="Q24" s="32"/>
       <c r="R24" s="49">
         <f t="shared" ref="R24:X24" si="1">SUM(R23:R23)</f>
-        <v>13.72</v>
+        <v>34.3</v>
       </c>
       <c r="S24" s="50">
         <f t="shared" si="1"/>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="T24" s="49"/>
       <c r="U24" s="49"/>
@@ -10969,7 +10975,7 @@
       </c>
       <c r="AC24" s="52">
         <f t="shared" si="2"/>
-        <v>186.28</v>
+        <v>465.7</v>
       </c>
       <c r="AD24" s="53">
         <f t="shared" si="2"/>
@@ -10990,7 +10996,7 @@
       </c>
       <c r="AI24" s="53">
         <f t="shared" si="3"/>
-        <v>15833.8</v>
+        <v>39584.5</v>
       </c>
       <c r="AJ24" s="53">
         <f t="shared" si="3"/>
@@ -17583,7 +17589,7 @@
       <c r="BP21" s="33"/>
       <c r="BQ21" s="33"/>
     </row>
-    <row r="22" s="55" customFormat="1" ht="15.25" spans="1:69">
+    <row r="22" s="56" customFormat="1" ht="15.25" spans="1:69">
       <c r="A22" s="34" t="s">
         <v>2</v>
       </c>
@@ -17776,10 +17782,10 @@
       <c r="BL22" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="BM22" s="56" t="s">
+      <c r="BM22" s="57" t="s">
         <v>144</v>
       </c>
-      <c r="BN22" s="56" t="s">
+      <c r="BN22" s="57" t="s">
         <v>145</v>
       </c>
       <c r="BO22" s="34" t="s">
@@ -20166,10 +20172,10 @@
       <c r="A23" s="28">
         <v>1</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="55" t="s">
         <v>150</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="55" t="s">
         <v>150</v>
       </c>
       <c r="D23" s="28" t="s">
@@ -20182,11 +20188,11 @@
         <v>3</v>
       </c>
       <c r="G23" s="41">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="H23" s="42">
         <f>F23*G23</f>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="I23" s="43">
         <v>1</v>
@@ -20199,35 +20205,35 @@
       </c>
       <c r="L23" s="42">
         <f>H23</f>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="M23" s="42">
         <f>ROUND(L23*I23%,2)</f>
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="N23" s="42">
         <f>H23-M23</f>
-        <v>297</v>
+        <v>742.5</v>
       </c>
       <c r="O23" s="42">
         <f>ROUND(N23*J23%,2)</f>
-        <v>5.94</v>
+        <v>14.85</v>
       </c>
       <c r="P23" s="42">
         <f>ROUND(N23-O23,2)</f>
-        <v>291.06</v>
+        <v>727.65</v>
       </c>
       <c r="Q23" s="42">
         <f>ROUND(P23*K23%,2)</f>
-        <v>11.64</v>
+        <v>29.11</v>
       </c>
       <c r="R23" s="42">
         <f>M23+O23+Q23</f>
-        <v>20.58</v>
+        <v>51.46</v>
       </c>
       <c r="S23" s="42">
         <f>(H23-R23)</f>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="T23" s="42" t="s">
         <v>107</v>
@@ -20264,7 +20270,7 @@
       </c>
       <c r="AC23" s="42">
         <f>IF($V21=1,S23+AB23,S23)</f>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="AD23" s="42">
         <v>120</v>
@@ -20284,7 +20290,7 @@
       </c>
       <c r="AI23" s="42">
         <f>S23*$M$21</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AJ23" s="42">
         <f>IF($C$21=3,0,AG23+AH23)</f>
@@ -20303,7 +20309,7 @@
       </c>
       <c r="AN23" s="42">
         <f>AI23/AM23</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AO23" s="42">
         <f>AJ23/AM23</f>
@@ -20318,7 +20324,7 @@
       </c>
       <c r="AR23" s="42">
         <f>AN23+AO23+AP23</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AS23" s="42" t="s">
         <v>108</v>
@@ -20338,7 +20344,7 @@
       </c>
       <c r="AX23" s="42">
         <f>AR23</f>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AY23" s="42">
         <f>AU23+AW23</f>
@@ -20399,7 +20405,7 @@
       <c r="G24" s="49"/>
       <c r="H24" s="49">
         <f>SUM(H23:H23)</f>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -20412,11 +20418,11 @@
       <c r="Q24" s="32"/>
       <c r="R24" s="49">
         <f t="shared" ref="R24:Y24" si="1">SUM(R23:R23)</f>
-        <v>20.58</v>
+        <v>51.46</v>
       </c>
       <c r="S24" s="50">
         <f t="shared" si="1"/>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="T24" s="49"/>
       <c r="U24" s="49"/>
@@ -20447,7 +20453,7 @@
       </c>
       <c r="AC24" s="52">
         <f t="shared" si="2"/>
-        <v>279.42</v>
+        <v>698.54</v>
       </c>
       <c r="AD24" s="53">
         <f t="shared" si="2"/>
@@ -20468,7 +20474,7 @@
       </c>
       <c r="AI24" s="53">
         <f t="shared" si="3"/>
-        <v>23750.7</v>
+        <v>59375.9</v>
       </c>
       <c r="AJ24" s="53">
         <f t="shared" si="3"/>

</xml_diff>